<commit_message>
Revision de planos: murete en el escalon de ambas cajas (plantas, cortes, perfil, isometrico, metrado), barras a diametro real, acero dentro del concreto, llamadas ordenadas
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_PLUVIAL_MUJERES_VIOLENTADAS_CON_COLECTOR.xlsx
+++ b/entregables/METRADO_DRENAJE_PLUVIAL_MUJERES_VIOLENTADAS_CON_COLECTOR.xlsx
@@ -7846,7 +7846,7 @@
         <v>0.351</v>
       </c>
       <c r="I34" s="366" t="n">
-        <v>1.26</v>
+        <v>1.305</v>
       </c>
       <c r="J34" s="366" t="n">
         <v>0.185</v>
@@ -7880,7 +7880,7 @@
         <v>2.18</v>
       </c>
       <c r="E35" s="366" t="n">
-        <v>1.521</v>
+        <v>1.576</v>
       </c>
       <c r="F35" s="367">
         <f>(B35+2*$B$6+2*$B$11)*(C35+2*$B$6+2*$B$11)*E35</f>
@@ -7891,22 +7891,22 @@
         <v/>
       </c>
       <c r="H35" s="366" t="n">
-        <v>1.135</v>
+        <v>1.176</v>
       </c>
       <c r="I35" s="366" t="n">
-        <v>2.688</v>
+        <v>2.915</v>
       </c>
       <c r="J35" s="366" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.586</v>
       </c>
       <c r="K35" s="366" t="n">
-        <v>50.05</v>
+        <v>50.91</v>
       </c>
       <c r="L35" s="366" t="n">
-        <v>206.8</v>
+        <v>208.6</v>
       </c>
       <c r="M35" s="366" t="n">
-        <v>6.57</v>
+        <v>6.84</v>
       </c>
       <c r="N35" s="366" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Metrado: la prolongacion de las cunetas de los Ejes 11 y 12 sale de la partida 01.04.04 (queda en cunetas de arquitectura, solo nota); leyenda con simbolo de flujo a escala de papel
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_PLUVIAL_MUJERES_VIOLENTADAS_CON_COLECTOR.xlsx
+++ b/entregables/METRADO_DRENAJE_PLUVIAL_MUJERES_VIOLENTADAS_CON_COLECTOR.xlsx
@@ -2977,7 +2977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.54296875" defaultRowHeight="15.5"/>
   <cols>
     <col width="18.08984375" customWidth="1" style="26" min="1" max="1"/>
@@ -3992,7 +3992,7 @@
         </is>
       </c>
       <c r="D57" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K197</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K195</f>
         <v/>
       </c>
     </row>
@@ -4013,7 +4013,7 @@
         </is>
       </c>
       <c r="D58" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K207</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K205</f>
         <v/>
       </c>
     </row>
@@ -4034,7 +4034,7 @@
         </is>
       </c>
       <c r="D59" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K224</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K222</f>
         <v/>
       </c>
     </row>
@@ -4069,7 +4069,7 @@
         </is>
       </c>
       <c r="D61" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K228</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K226</f>
         <v/>
       </c>
     </row>
@@ -4104,7 +4104,7 @@
         </is>
       </c>
       <c r="D63" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K241</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K237</f>
         <v/>
       </c>
     </row>
@@ -4125,7 +4125,7 @@
         </is>
       </c>
       <c r="D64" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K251</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K247</f>
         <v/>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
         </is>
       </c>
       <c r="D65" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K261</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K257</f>
         <v/>
       </c>
     </row>
@@ -4167,7 +4167,7 @@
         </is>
       </c>
       <c r="D66" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K273</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K269</f>
         <v/>
       </c>
     </row>
@@ -4188,7 +4188,7 @@
         </is>
       </c>
       <c r="D67" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K283</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K279</f>
         <v/>
       </c>
     </row>
@@ -4209,7 +4209,7 @@
         </is>
       </c>
       <c r="D68" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K284</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K280</f>
         <v/>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
         </is>
       </c>
       <c r="D69" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K294</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K290</f>
         <v/>
       </c>
     </row>
@@ -4265,7 +4265,7 @@
         </is>
       </c>
       <c r="D71" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K298</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K294</f>
         <v/>
       </c>
     </row>
@@ -4286,7 +4286,7 @@
         </is>
       </c>
       <c r="D72" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K299</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K295</f>
         <v/>
       </c>
     </row>
@@ -4307,7 +4307,7 @@
         </is>
       </c>
       <c r="D73" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K300</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K296</f>
         <v/>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
         </is>
       </c>
       <c r="D74" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K301</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K297</f>
         <v/>
       </c>
     </row>
@@ -4349,7 +4349,7 @@
         </is>
       </c>
       <c r="D75" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K302</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K298</f>
         <v/>
       </c>
     </row>
@@ -4370,7 +4370,7 @@
         </is>
       </c>
       <c r="D76" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K303</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K299</f>
         <v/>
       </c>
     </row>
@@ -4391,7 +4391,7 @@
         </is>
       </c>
       <c r="D77" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K304</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K300</f>
         <v/>
       </c>
     </row>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="B78" s="158" t="inlineStr">
         <is>
-          <t>JUNTAS, EMPALMES Y PROLONGACION DE CUNETAS</t>
+          <t>JUNTAS Y EMPALMES</t>
         </is>
       </c>
       <c r="C78" s="158" t="n"/>
@@ -4426,7 +4426,7 @@
         </is>
       </c>
       <c r="D79" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K306</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K302</f>
         <v/>
       </c>
     </row>
@@ -4447,7 +4447,7 @@
         </is>
       </c>
       <c r="D80" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K308</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K304</f>
         <v/>
       </c>
     </row>
@@ -4468,91 +4468,7 @@
         </is>
       </c>
       <c r="D81" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K311</f>
-        <v/>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="159" t="inlineStr">
-        <is>
-          <t>01.04.04.06.04</t>
-        </is>
-      </c>
-      <c r="B82" s="160" t="inlineStr">
-        <is>
-          <t>CONCRETO f'c=210 kg/cm2 EN PROLONGACION DE CUNETAS 0.40 x H</t>
-        </is>
-      </c>
-      <c r="C82" s="161" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="D82" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K313</f>
-        <v/>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="159" t="inlineStr">
-        <is>
-          <t>01.04.04.06.05</t>
-        </is>
-      </c>
-      <c r="B83" s="160" t="inlineStr">
-        <is>
-          <t>ENCOFRADO Y DESENCOFRADO EN PROLONGACION DE CUNETAS</t>
-        </is>
-      </c>
-      <c r="C83" s="161" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D83" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K316</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="159" t="inlineStr">
-        <is>
-          <t>01.04.04.06.06</t>
-        </is>
-      </c>
-      <c r="B84" s="160" t="inlineStr">
-        <is>
-          <t>ACERO DE REFUERZO fy=4200 kg/cm2 EN PROLONGACION DE CUNETAS</t>
-        </is>
-      </c>
-      <c r="C84" s="161" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="D84" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K319</f>
-        <v/>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="159" t="inlineStr">
-        <is>
-          <t>01.04.04.06.07</t>
-        </is>
-      </c>
-      <c r="B85" s="160" t="inlineStr">
-        <is>
-          <t>TAPA DE CONCRETO EN PROLONGACION DE CUNETAS (losa 0.60 x 0.08)</t>
-        </is>
-      </c>
-      <c r="C85" s="161" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D85" s="162">
-        <f>+'PLANILLA GENERAL DE METRADOS'!K320</f>
+        <f>+'PLANILLA GENERAL DE METRADOS'!K307</f>
         <v/>
       </c>
     </row>
@@ -7740,7 +7656,7 @@
     <row r="32">
       <c r="A32" s="361" t="inlineStr">
         <is>
-          <t>CAJAS Y PROLONGACIONES DE CUNETA (geometria de las laminas DP-06C y DP-07)</t>
+          <t>CAJAS DE LLEGADA Y DE CAIDA (geometria de la lamina DP-07)</t>
         </is>
       </c>
     </row>
@@ -7912,88 +7828,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="367" t="inlineStr">
-        <is>
-          <t>Prolongacion cuneta Eje 11 (0.40 x H, muros 0.10)</t>
-        </is>
-      </c>
-      <c r="B36" s="366" t="n">
-        <v>1.88</v>
-      </c>
-      <c r="C36" s="366" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D36" s="366" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="E36" s="366" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="F36" s="367">
-        <f>0.90*B36*E36</f>
-        <v/>
-      </c>
-      <c r="G36" s="367">
-        <f>0.70*B36</f>
-        <v/>
-      </c>
-      <c r="I36" s="367">
-        <f>B36*(0.60*0.10+2*0.10*(D36-0.10))</f>
-        <v/>
-      </c>
-      <c r="K36" s="367">
-        <f>B36*(2*(D36-0.10)+2*D36)</f>
-        <v/>
-      </c>
-      <c r="L36" s="366" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="M36" s="367">
-        <f>0.60*B36</f>
-        <v/>
-      </c>
-    </row>
     <row r="37">
-      <c r="A37" s="367" t="inlineStr">
-        <is>
-          <t>Prolongacion cuneta Eje 12 (0.40 x H, muros 0.10)</t>
-        </is>
-      </c>
-      <c r="B37" s="366" t="n">
-        <v>5.39</v>
-      </c>
-      <c r="C37" s="366" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D37" s="366" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E37" s="366" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="F37" s="367">
-        <f>0.90*B37*E37</f>
-        <v/>
-      </c>
-      <c r="G37" s="367">
-        <f>0.70*B37</f>
-        <v/>
-      </c>
-      <c r="I37" s="367">
-        <f>B37*(0.60*0.10+2*0.10*(D37-0.10))</f>
-        <v/>
-      </c>
-      <c r="K37" s="367">
-        <f>B37*(2*(D37-0.10)+2*D37)</f>
-        <v/>
-      </c>
-      <c r="L37" s="366" t="n">
-        <v>75.40000000000001</v>
-      </c>
-      <c r="M37" s="367">
-        <f>0.60*B37</f>
-        <v/>
+      <c r="A37" s="362" t="inlineStr">
+        <is>
+          <t>NOTA: las cunetas de los Ejes 11 y 12 (perfiles 11 y 12) se prolongan 1.88 m y 5.39 m hasta el muro del colector con su misma seccion 0.40 x H. Esa prolongacion NO forma parte de la partida 01.04.04: se metra dentro de las partidas de cunetas del proyecto (arquitectura). Aqui solo se metra la ventana de empalme (partida 01.04.04.06.03).</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -8007,7 +7846,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -8329,81 +8168,36 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="365" t="inlineStr">
-        <is>
-          <t>Prolongacion de cunetas Ejes 11 y 12</t>
-        </is>
-      </c>
-      <c r="B11" s="365" t="inlineStr">
-        <is>
-          <t>3/8"</t>
-        </is>
-      </c>
-      <c r="C11" s="365" t="inlineStr">
-        <is>
-          <t>U + rectas</t>
-        </is>
-      </c>
-      <c r="F11" s="367">
-        <f>('COLECTOR TRAMOS'!L36+'COLECTOR TRAMOS'!L37)/'COLECTOR TRAMOS'!$B$14</f>
-        <v/>
-      </c>
-      <c r="G11" s="367">
-        <f>'COLECTOR TRAMOS'!$B$14</f>
-        <v/>
-      </c>
-      <c r="H11" s="367">
-        <f>F11*G11</f>
-        <v/>
-      </c>
-      <c r="I11" s="365" t="inlineStr">
-        <is>
-          <t>@0.20</t>
-        </is>
+    <row r="12">
+      <c r="A12" s="361" t="inlineStr">
+        <is>
+          <t>TOTAL ACERO COLECTOR Y CAJAS (partida 01.04.04.04.05)</t>
+        </is>
+      </c>
+      <c r="H12" s="371">
+        <f>SUM(H4:H6)</f>
+        <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="361" t="inlineStr">
         <is>
-          <t>TOTAL ACERO COLECTOR Y CAJAS (partida 01.04.04.04.05)</t>
+          <t>TOTAL ACERO EN REGISTROS Y TAPAS (partida 01.04.04.05.06)</t>
         </is>
       </c>
       <c r="H13" s="371">
-        <f>SUM(H4:H6)</f>
+        <f>SUM(H7:H10)</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="361" t="inlineStr">
         <is>
-          <t>TOTAL ACERO EN REGISTROS Y TAPAS (partida 01.04.04.05.06)</t>
+          <t>TOTAL ACERO</t>
         </is>
       </c>
       <c r="H14" s="371">
-        <f>SUM(H7:H10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="361" t="inlineStr">
-        <is>
-          <t>TOTAL ACERO EN PROLONGACION DE CUNETAS (partida 01.04.04.06.06)</t>
-        </is>
-      </c>
-      <c r="H15" s="371">
-        <f>H11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="361" t="inlineStr">
-        <is>
-          <t>TOTAL ACERO</t>
-        </is>
-      </c>
-      <c r="H16" s="371">
-        <f>SUM(H4:H11)</f>
+        <f>SUM(H4:H10)</f>
         <v/>
       </c>
     </row>
@@ -8874,7 +8668,7 @@
         </is>
       </c>
       <c r="C5" s="367">
-        <f>'PLANILLA GENERAL DE METRADOS'!K241</f>
+        <f>'PLANILLA GENERAL DE METRADOS'!K237</f>
         <v/>
       </c>
       <c r="D5" s="365" t="inlineStr">
@@ -9083,7 +8877,7 @@
         </is>
       </c>
       <c r="C15" s="367">
-        <f>'PLANILLA GENERAL DE METRADOS'!K251</f>
+        <f>'PLANILLA GENERAL DE METRADOS'!K247</f>
         <v/>
       </c>
       <c r="D15" s="365" t="inlineStr">
@@ -9292,7 +9086,7 @@
         </is>
       </c>
       <c r="C25" s="367">
-        <f>'PLANILLA GENERAL DE METRADOS'!K261</f>
+        <f>'PLANILLA GENERAL DE METRADOS'!K257</f>
         <v/>
       </c>
       <c r="D25" s="365" t="inlineStr">
@@ -9501,7 +9295,7 @@
         </is>
       </c>
       <c r="C35" s="367">
-        <f>'PLANILLA GENERAL DE METRADOS'!K273</f>
+        <f>'PLANILLA GENERAL DE METRADOS'!K269</f>
         <v/>
       </c>
       <c r="D35" s="365" t="inlineStr">
@@ -9622,7 +9416,7 @@
         </is>
       </c>
       <c r="C41" s="367">
-        <f>'PLANILLA GENERAL DE METRADOS'!K283</f>
+        <f>'PLANILLA GENERAL DE METRADOS'!K279</f>
         <v/>
       </c>
       <c r="D41" s="365" t="inlineStr">
@@ -9721,7 +9515,7 @@
         </is>
       </c>
       <c r="C46" s="367">
-        <f>'PLANILLA GENERAL DE METRADOS'!K228</f>
+        <f>'PLANILLA GENERAL DE METRADOS'!K226</f>
         <v/>
       </c>
       <c r="D46" s="365" t="inlineStr">
@@ -9897,7 +9691,7 @@
         </is>
       </c>
       <c r="C55" s="367">
-        <f>'PLANILLA GENERAL DE METRADOS'!K207</f>
+        <f>'PLANILLA GENERAL DE METRADOS'!K205</f>
         <v/>
       </c>
       <c r="D55" s="365" t="inlineStr">
@@ -9996,7 +9790,7 @@
         </is>
       </c>
       <c r="C60" s="367">
-        <f>'PLANILLA GENERAL DE METRADOS'!K224</f>
+        <f>'PLANILLA GENERAL DE METRADOS'!K222</f>
         <v/>
       </c>
       <c r="D60" s="365" t="inlineStr">
@@ -10073,7 +9867,7 @@
         </is>
       </c>
       <c r="C64" s="367">
-        <f>'PLANILLA GENERAL DE METRADOS'!K300</f>
+        <f>'PLANILLA GENERAL DE METRADOS'!K296</f>
         <v/>
       </c>
       <c r="D64" s="365" t="inlineStr">
@@ -10172,7 +9966,7 @@
         </is>
       </c>
       <c r="C69" s="367">
-        <f>'PLANILLA GENERAL DE METRADOS'!K304</f>
+        <f>'PLANILLA GENERAL DE METRADOS'!K300</f>
         <v/>
       </c>
       <c r="D69" s="365" t="inlineStr">
@@ -10271,7 +10065,7 @@
         </is>
       </c>
       <c r="C74" s="367">
-        <f>'PLANILLA GENERAL DE METRADOS'!K306</f>
+        <f>'PLANILLA GENERAL DE METRADOS'!K302</f>
         <v/>
       </c>
       <c r="D74" s="365" t="inlineStr">
@@ -10370,7 +10164,7 @@
         </is>
       </c>
       <c r="C79" s="367">
-        <f>'PLANILLA GENERAL DE METRADOS'!K308</f>
+        <f>'PLANILLA GENERAL DE METRADOS'!K304</f>
         <v/>
       </c>
       <c r="D79" s="365" t="inlineStr">
@@ -10424,7 +10218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L322"/>
+  <dimension ref="A1:L308"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col width="18.81640625" customWidth="1" min="1" max="1"/>
@@ -15153,7 +14947,7 @@
       <c r="I185" s="29" t="n"/>
       <c r="J185" s="29" t="n"/>
       <c r="K185" s="29">
-        <f>SUM(J186:J196)</f>
+        <f>SUM(J186:J194)</f>
         <v/>
       </c>
       <c r="L185" s="28" t="inlineStr">
@@ -15370,33 +15164,39 @@
       <c r="L194" s="30" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" s="30" t="n"/>
-      <c r="B195" s="30" t="inlineStr">
-        <is>
-          <t>Prolongacion cuneta Eje 11</t>
-        </is>
-      </c>
-      <c r="C195" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D195" s="31" t="n"/>
-      <c r="E195" s="31" t="n"/>
-      <c r="F195" s="31" t="n"/>
-      <c r="G195" s="31" t="n"/>
-      <c r="H195" s="31" t="n"/>
-      <c r="I195" s="31" t="n"/>
-      <c r="J195" s="31">
-        <f>'COLECTOR TRAMOS'!F36</f>
-        <v/>
-      </c>
-      <c r="K195" s="31" t="n"/>
-      <c r="L195" s="30" t="n"/>
+      <c r="A195" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.02.02</t>
+        </is>
+      </c>
+      <c r="B195" s="28" t="inlineStr">
+        <is>
+          <t>REFINE, NIVELACIÓN Y COMPACTACIÓN EN TERRENO NORMAL</t>
+        </is>
+      </c>
+      <c r="C195" s="29" t="n"/>
+      <c r="D195" s="29" t="n"/>
+      <c r="E195" s="29" t="n"/>
+      <c r="F195" s="29" t="n"/>
+      <c r="G195" s="29" t="n"/>
+      <c r="H195" s="29" t="n"/>
+      <c r="I195" s="29" t="n"/>
+      <c r="J195" s="29" t="n"/>
+      <c r="K195" s="29">
+        <f>SUM(J196:J204)</f>
+        <v/>
+      </c>
+      <c r="L195" s="28" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="30" t="n"/>
       <c r="B196" s="30" t="inlineStr">
         <is>
-          <t>Prolongacion cuneta Eje 12</t>
+          <t>Tramo normal (0+000.00 - 0+026.32)</t>
         </is>
       </c>
       <c r="C196" s="31" t="n">
@@ -15409,46 +15209,40 @@
       <c r="H196" s="31" t="n"/>
       <c r="I196" s="31" t="n"/>
       <c r="J196" s="31">
-        <f>'COLECTOR TRAMOS'!F37</f>
+        <f>'COLECTOR TRAMOS'!N22</f>
         <v/>
       </c>
       <c r="K196" s="31" t="n"/>
       <c r="L196" s="30" t="n"/>
     </row>
     <row r="197">
-      <c r="A197" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.02.02</t>
-        </is>
-      </c>
-      <c r="B197" s="28" t="inlineStr">
-        <is>
-          <t>REFINE, NIVELACIÓN Y COMPACTACIÓN EN TERRENO NORMAL</t>
-        </is>
-      </c>
-      <c r="C197" s="29" t="n"/>
-      <c r="D197" s="29" t="n"/>
-      <c r="E197" s="29" t="n"/>
-      <c r="F197" s="29" t="n"/>
-      <c r="G197" s="29" t="n"/>
-      <c r="H197" s="29" t="n"/>
-      <c r="I197" s="29" t="n"/>
-      <c r="J197" s="29" t="n"/>
-      <c r="K197" s="29">
-        <f>SUM(J198:J206)</f>
-        <v/>
-      </c>
-      <c r="L197" s="28" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
+      <c r="A197" s="30" t="n"/>
+      <c r="B197" s="30" t="inlineStr">
+        <is>
+          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
+        </is>
+      </c>
+      <c r="C197" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D197" s="31" t="n"/>
+      <c r="E197" s="31" t="n"/>
+      <c r="F197" s="31" t="n"/>
+      <c r="G197" s="31" t="n"/>
+      <c r="H197" s="31" t="n"/>
+      <c r="I197" s="31" t="n"/>
+      <c r="J197" s="31">
+        <f>'COLECTOR TRAMOS'!N23</f>
+        <v/>
+      </c>
+      <c r="K197" s="31" t="n"/>
+      <c r="L197" s="30" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="30" t="n"/>
       <c r="B198" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+000.00 - 0+026.32)</t>
+          <t>Tramo normal (0+031.33 - 0+039.04)</t>
         </is>
       </c>
       <c r="C198" s="31" t="n">
@@ -15461,7 +15255,7 @@
       <c r="H198" s="31" t="n"/>
       <c r="I198" s="31" t="n"/>
       <c r="J198" s="31">
-        <f>'COLECTOR TRAMOS'!N22</f>
+        <f>'COLECTOR TRAMOS'!N24</f>
         <v/>
       </c>
       <c r="K198" s="31" t="n"/>
@@ -15471,7 +15265,7 @@
       <c r="A199" s="30" t="n"/>
       <c r="B199" s="30" t="inlineStr">
         <is>
-          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
+          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
         </is>
       </c>
       <c r="C199" s="31" t="n">
@@ -15484,7 +15278,7 @@
       <c r="H199" s="31" t="n"/>
       <c r="I199" s="31" t="n"/>
       <c r="J199" s="31">
-        <f>'COLECTOR TRAMOS'!N23</f>
+        <f>'COLECTOR TRAMOS'!N25</f>
         <v/>
       </c>
       <c r="K199" s="31" t="n"/>
@@ -15494,7 +15288,7 @@
       <c r="A200" s="30" t="n"/>
       <c r="B200" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+031.33 - 0+039.04)</t>
+          <t>Tramo normal (0+041.04 - 0+058.81)</t>
         </is>
       </c>
       <c r="C200" s="31" t="n">
@@ -15507,7 +15301,7 @@
       <c r="H200" s="31" t="n"/>
       <c r="I200" s="31" t="n"/>
       <c r="J200" s="31">
-        <f>'COLECTOR TRAMOS'!N24</f>
+        <f>'COLECTOR TRAMOS'!N26</f>
         <v/>
       </c>
       <c r="K200" s="31" t="n"/>
@@ -15517,7 +15311,7 @@
       <c r="A201" s="30" t="n"/>
       <c r="B201" s="30" t="inlineStr">
         <is>
-          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
+          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
         </is>
       </c>
       <c r="C201" s="31" t="n">
@@ -15530,7 +15324,7 @@
       <c r="H201" s="31" t="n"/>
       <c r="I201" s="31" t="n"/>
       <c r="J201" s="31">
-        <f>'COLECTOR TRAMOS'!N25</f>
+        <f>'COLECTOR TRAMOS'!N27</f>
         <v/>
       </c>
       <c r="K201" s="31" t="n"/>
@@ -15540,7 +15334,7 @@
       <c r="A202" s="30" t="n"/>
       <c r="B202" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+041.04 - 0+058.81)</t>
+          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
         </is>
       </c>
       <c r="C202" s="31" t="n">
@@ -15553,7 +15347,7 @@
       <c r="H202" s="31" t="n"/>
       <c r="I202" s="31" t="n"/>
       <c r="J202" s="31">
-        <f>'COLECTOR TRAMOS'!N26</f>
+        <f>'COLECTOR TRAMOS'!N28</f>
         <v/>
       </c>
       <c r="K202" s="31" t="n"/>
@@ -15563,7 +15357,7 @@
       <c r="A203" s="30" t="n"/>
       <c r="B203" s="30" t="inlineStr">
         <is>
-          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
+          <t>Caja de llegada CL</t>
         </is>
       </c>
       <c r="C203" s="31" t="n">
@@ -15576,7 +15370,7 @@
       <c r="H203" s="31" t="n"/>
       <c r="I203" s="31" t="n"/>
       <c r="J203" s="31">
-        <f>'COLECTOR TRAMOS'!N27</f>
+        <f>'COLECTOR TRAMOS'!G34</f>
         <v/>
       </c>
       <c r="K203" s="31" t="n"/>
@@ -15586,7 +15380,7 @@
       <c r="A204" s="30" t="n"/>
       <c r="B204" s="30" t="inlineStr">
         <is>
-          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
+          <t>Caja de caida CC</t>
         </is>
       </c>
       <c r="C204" s="31" t="n">
@@ -15599,40 +15393,46 @@
       <c r="H204" s="31" t="n"/>
       <c r="I204" s="31" t="n"/>
       <c r="J204" s="31">
-        <f>'COLECTOR TRAMOS'!N28</f>
+        <f>'COLECTOR TRAMOS'!G35</f>
         <v/>
       </c>
       <c r="K204" s="31" t="n"/>
       <c r="L204" s="30" t="n"/>
     </row>
     <row r="205">
-      <c r="A205" s="30" t="n"/>
-      <c r="B205" s="30" t="inlineStr">
-        <is>
-          <t>Caja de llegada CL</t>
-        </is>
-      </c>
-      <c r="C205" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D205" s="31" t="n"/>
-      <c r="E205" s="31" t="n"/>
-      <c r="F205" s="31" t="n"/>
-      <c r="G205" s="31" t="n"/>
-      <c r="H205" s="31" t="n"/>
-      <c r="I205" s="31" t="n"/>
-      <c r="J205" s="31">
-        <f>'COLECTOR TRAMOS'!G34</f>
-        <v/>
-      </c>
-      <c r="K205" s="31" t="n"/>
-      <c r="L205" s="30" t="n"/>
+      <c r="A205" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.02.03</t>
+        </is>
+      </c>
+      <c r="B205" s="28" t="inlineStr">
+        <is>
+          <t>RELLENO COMPACTADO CON MATERIAL PROPIO SELECCIONADO (incluye nivelacion del retiro y base de cajas)</t>
+        </is>
+      </c>
+      <c r="C205" s="29" t="n"/>
+      <c r="D205" s="29" t="n"/>
+      <c r="E205" s="29" t="n"/>
+      <c r="F205" s="29" t="n"/>
+      <c r="G205" s="29" t="n"/>
+      <c r="H205" s="29" t="n"/>
+      <c r="I205" s="29" t="n"/>
+      <c r="J205" s="29" t="n"/>
+      <c r="K205" s="29">
+        <f>SUM(J206:J221)</f>
+        <v/>
+      </c>
+      <c r="L205" s="28" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="30" t="n"/>
       <c r="B206" s="30" t="inlineStr">
         <is>
-          <t>Caja de caida CC</t>
+          <t>Tramo normal (0+000.00 - 0+026.32) - lateral de zanja</t>
         </is>
       </c>
       <c r="C206" s="31" t="n">
@@ -15645,46 +15445,40 @@
       <c r="H206" s="31" t="n"/>
       <c r="I206" s="31" t="n"/>
       <c r="J206" s="31">
-        <f>'COLECTOR TRAMOS'!G35</f>
+        <f>'COLECTOR TRAMOS'!O22</f>
         <v/>
       </c>
       <c r="K206" s="31" t="n"/>
       <c r="L206" s="30" t="n"/>
     </row>
     <row r="207">
-      <c r="A207" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.02.03</t>
-        </is>
-      </c>
-      <c r="B207" s="28" t="inlineStr">
-        <is>
-          <t>RELLENO COMPACTADO CON MATERIAL PROPIO SELECCIONADO (incluye nivelacion del retiro y base de cajas)</t>
-        </is>
-      </c>
-      <c r="C207" s="29" t="n"/>
-      <c r="D207" s="29" t="n"/>
-      <c r="E207" s="29" t="n"/>
-      <c r="F207" s="29" t="n"/>
-      <c r="G207" s="29" t="n"/>
-      <c r="H207" s="29" t="n"/>
-      <c r="I207" s="29" t="n"/>
-      <c r="J207" s="29" t="n"/>
-      <c r="K207" s="29">
-        <f>SUM(J208:J223)</f>
-        <v/>
-      </c>
-      <c r="L207" s="28" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
+      <c r="A207" s="30" t="n"/>
+      <c r="B207" s="30" t="inlineStr">
+        <is>
+          <t>Cruce de camiones (0+026.32 - 0+031.33) - lateral de zanja</t>
+        </is>
+      </c>
+      <c r="C207" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D207" s="31" t="n"/>
+      <c r="E207" s="31" t="n"/>
+      <c r="F207" s="31" t="n"/>
+      <c r="G207" s="31" t="n"/>
+      <c r="H207" s="31" t="n"/>
+      <c r="I207" s="31" t="n"/>
+      <c r="J207" s="31">
+        <f>'COLECTOR TRAMOS'!O23</f>
+        <v/>
+      </c>
+      <c r="K207" s="31" t="n"/>
+      <c r="L207" s="30" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="30" t="n"/>
       <c r="B208" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+000.00 - 0+026.32) - lateral de zanja</t>
+          <t>Tramo normal (0+031.33 - 0+039.04) - lateral de zanja</t>
         </is>
       </c>
       <c r="C208" s="31" t="n">
@@ -15697,7 +15491,7 @@
       <c r="H208" s="31" t="n"/>
       <c r="I208" s="31" t="n"/>
       <c r="J208" s="31">
-        <f>'COLECTOR TRAMOS'!O22</f>
+        <f>'COLECTOR TRAMOS'!O24</f>
         <v/>
       </c>
       <c r="K208" s="31" t="n"/>
@@ -15707,7 +15501,7 @@
       <c r="A209" s="30" t="n"/>
       <c r="B209" s="30" t="inlineStr">
         <is>
-          <t>Cruce de camiones (0+026.32 - 0+031.33) - lateral de zanja</t>
+          <t>Cruce de motos (0+039.04 - 0+041.04) - lateral de zanja</t>
         </is>
       </c>
       <c r="C209" s="31" t="n">
@@ -15720,7 +15514,7 @@
       <c r="H209" s="31" t="n"/>
       <c r="I209" s="31" t="n"/>
       <c r="J209" s="31">
-        <f>'COLECTOR TRAMOS'!O23</f>
+        <f>'COLECTOR TRAMOS'!O25</f>
         <v/>
       </c>
       <c r="K209" s="31" t="n"/>
@@ -15730,7 +15524,7 @@
       <c r="A210" s="30" t="n"/>
       <c r="B210" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+031.33 - 0+039.04) - lateral de zanja</t>
+          <t>Tramo normal (0+041.04 - 0+058.81) - lateral de zanja</t>
         </is>
       </c>
       <c r="C210" s="31" t="n">
@@ -15743,7 +15537,7 @@
       <c r="H210" s="31" t="n"/>
       <c r="I210" s="31" t="n"/>
       <c r="J210" s="31">
-        <f>'COLECTOR TRAMOS'!O24</f>
+        <f>'COLECTOR TRAMOS'!O26</f>
         <v/>
       </c>
       <c r="K210" s="31" t="n"/>
@@ -15753,7 +15547,7 @@
       <c r="A211" s="30" t="n"/>
       <c r="B211" s="30" t="inlineStr">
         <is>
-          <t>Cruce de motos (0+039.04 - 0+041.04) - lateral de zanja</t>
+          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89) - lateral de zanja</t>
         </is>
       </c>
       <c r="C211" s="31" t="n">
@@ -15766,7 +15560,7 @@
       <c r="H211" s="31" t="n"/>
       <c r="I211" s="31" t="n"/>
       <c r="J211" s="31">
-        <f>'COLECTOR TRAMOS'!O25</f>
+        <f>'COLECTOR TRAMOS'!O27</f>
         <v/>
       </c>
       <c r="K211" s="31" t="n"/>
@@ -15776,7 +15570,7 @@
       <c r="A212" s="30" t="n"/>
       <c r="B212" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+041.04 - 0+058.81) - lateral de zanja</t>
+          <t>Tramo recto final (0+066.89 - 0+069.89) - lateral de zanja</t>
         </is>
       </c>
       <c r="C212" s="31" t="n">
@@ -15789,7 +15583,7 @@
       <c r="H212" s="31" t="n"/>
       <c r="I212" s="31" t="n"/>
       <c r="J212" s="31">
-        <f>'COLECTOR TRAMOS'!O26</f>
+        <f>'COLECTOR TRAMOS'!O28</f>
         <v/>
       </c>
       <c r="K212" s="31" t="n"/>
@@ -15799,7 +15593,7 @@
       <c r="A213" s="30" t="n"/>
       <c r="B213" s="30" t="inlineStr">
         <is>
-          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89) - lateral de zanja</t>
+          <t>Tramo normal (0+000.00 - 0+026.32) - franja de nivelacion</t>
         </is>
       </c>
       <c r="C213" s="31" t="n">
@@ -15812,7 +15606,7 @@
       <c r="H213" s="31" t="n"/>
       <c r="I213" s="31" t="n"/>
       <c r="J213" s="31">
-        <f>'COLECTOR TRAMOS'!O27</f>
+        <f>'COLECTOR TRAMOS'!P22</f>
         <v/>
       </c>
       <c r="K213" s="31" t="n"/>
@@ -15822,7 +15616,7 @@
       <c r="A214" s="30" t="n"/>
       <c r="B214" s="30" t="inlineStr">
         <is>
-          <t>Tramo recto final (0+066.89 - 0+069.89) - lateral de zanja</t>
+          <t>Cruce de camiones (0+026.32 - 0+031.33) - franja de nivelacion</t>
         </is>
       </c>
       <c r="C214" s="31" t="n">
@@ -15835,7 +15629,7 @@
       <c r="H214" s="31" t="n"/>
       <c r="I214" s="31" t="n"/>
       <c r="J214" s="31">
-        <f>'COLECTOR TRAMOS'!O28</f>
+        <f>'COLECTOR TRAMOS'!P23</f>
         <v/>
       </c>
       <c r="K214" s="31" t="n"/>
@@ -15845,7 +15639,7 @@
       <c r="A215" s="30" t="n"/>
       <c r="B215" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+000.00 - 0+026.32) - franja de nivelacion</t>
+          <t>Tramo normal (0+031.33 - 0+039.04) - franja de nivelacion</t>
         </is>
       </c>
       <c r="C215" s="31" t="n">
@@ -15858,7 +15652,7 @@
       <c r="H215" s="31" t="n"/>
       <c r="I215" s="31" t="n"/>
       <c r="J215" s="31">
-        <f>'COLECTOR TRAMOS'!P22</f>
+        <f>'COLECTOR TRAMOS'!P24</f>
         <v/>
       </c>
       <c r="K215" s="31" t="n"/>
@@ -15868,7 +15662,7 @@
       <c r="A216" s="30" t="n"/>
       <c r="B216" s="30" t="inlineStr">
         <is>
-          <t>Cruce de camiones (0+026.32 - 0+031.33) - franja de nivelacion</t>
+          <t>Cruce de motos (0+039.04 - 0+041.04) - franja de nivelacion</t>
         </is>
       </c>
       <c r="C216" s="31" t="n">
@@ -15881,7 +15675,7 @@
       <c r="H216" s="31" t="n"/>
       <c r="I216" s="31" t="n"/>
       <c r="J216" s="31">
-        <f>'COLECTOR TRAMOS'!P23</f>
+        <f>'COLECTOR TRAMOS'!P25</f>
         <v/>
       </c>
       <c r="K216" s="31" t="n"/>
@@ -15891,7 +15685,7 @@
       <c r="A217" s="30" t="n"/>
       <c r="B217" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+031.33 - 0+039.04) - franja de nivelacion</t>
+          <t>Tramo normal (0+041.04 - 0+058.81) - franja de nivelacion</t>
         </is>
       </c>
       <c r="C217" s="31" t="n">
@@ -15904,7 +15698,7 @@
       <c r="H217" s="31" t="n"/>
       <c r="I217" s="31" t="n"/>
       <c r="J217" s="31">
-        <f>'COLECTOR TRAMOS'!P24</f>
+        <f>'COLECTOR TRAMOS'!P26</f>
         <v/>
       </c>
       <c r="K217" s="31" t="n"/>
@@ -15914,7 +15708,7 @@
       <c r="A218" s="30" t="n"/>
       <c r="B218" s="30" t="inlineStr">
         <is>
-          <t>Cruce de motos (0+039.04 - 0+041.04) - franja de nivelacion</t>
+          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89) - franja de nivelacion</t>
         </is>
       </c>
       <c r="C218" s="31" t="n">
@@ -15927,7 +15721,7 @@
       <c r="H218" s="31" t="n"/>
       <c r="I218" s="31" t="n"/>
       <c r="J218" s="31">
-        <f>'COLECTOR TRAMOS'!P25</f>
+        <f>'COLECTOR TRAMOS'!P27</f>
         <v/>
       </c>
       <c r="K218" s="31" t="n"/>
@@ -15937,7 +15731,7 @@
       <c r="A219" s="30" t="n"/>
       <c r="B219" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+041.04 - 0+058.81) - franja de nivelacion</t>
+          <t>Tramo recto final (0+066.89 - 0+069.89) - franja de nivelacion</t>
         </is>
       </c>
       <c r="C219" s="31" t="n">
@@ -15950,7 +15744,7 @@
       <c r="H219" s="31" t="n"/>
       <c r="I219" s="31" t="n"/>
       <c r="J219" s="31">
-        <f>'COLECTOR TRAMOS'!P26</f>
+        <f>'COLECTOR TRAMOS'!P28</f>
         <v/>
       </c>
       <c r="K219" s="31" t="n"/>
@@ -15960,7 +15754,7 @@
       <c r="A220" s="30" t="n"/>
       <c r="B220" s="30" t="inlineStr">
         <is>
-          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89) - franja de nivelacion</t>
+          <t>Caja de llegada CL</t>
         </is>
       </c>
       <c r="C220" s="31" t="n">
@@ -15973,7 +15767,7 @@
       <c r="H220" s="31" t="n"/>
       <c r="I220" s="31" t="n"/>
       <c r="J220" s="31">
-        <f>'COLECTOR TRAMOS'!P27</f>
+        <f>'COLECTOR TRAMOS'!N34</f>
         <v/>
       </c>
       <c r="K220" s="31" t="n"/>
@@ -15983,7 +15777,7 @@
       <c r="A221" s="30" t="n"/>
       <c r="B221" s="30" t="inlineStr">
         <is>
-          <t>Tramo recto final (0+066.89 - 0+069.89) - franja de nivelacion</t>
+          <t>Caja de caida CC</t>
         </is>
       </c>
       <c r="C221" s="31" t="n">
@@ -15996,40 +15790,46 @@
       <c r="H221" s="31" t="n"/>
       <c r="I221" s="31" t="n"/>
       <c r="J221" s="31">
-        <f>'COLECTOR TRAMOS'!P28</f>
+        <f>'COLECTOR TRAMOS'!N35</f>
         <v/>
       </c>
       <c r="K221" s="31" t="n"/>
       <c r="L221" s="30" t="n"/>
     </row>
     <row r="222">
-      <c r="A222" s="30" t="n"/>
-      <c r="B222" s="30" t="inlineStr">
-        <is>
-          <t>Caja de llegada CL</t>
-        </is>
-      </c>
-      <c r="C222" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D222" s="31" t="n"/>
-      <c r="E222" s="31" t="n"/>
-      <c r="F222" s="31" t="n"/>
-      <c r="G222" s="31" t="n"/>
-      <c r="H222" s="31" t="n"/>
-      <c r="I222" s="31" t="n"/>
-      <c r="J222" s="31">
-        <f>'COLECTOR TRAMOS'!N34</f>
-        <v/>
-      </c>
-      <c r="K222" s="31" t="n"/>
-      <c r="L222" s="30" t="n"/>
+      <c r="A222" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.02.04</t>
+        </is>
+      </c>
+      <c r="B222" s="28" t="inlineStr">
+        <is>
+          <t>ELIMINACIÓN DE MATERIAL EXCEDENTE</t>
+        </is>
+      </c>
+      <c r="C222" s="29" t="n"/>
+      <c r="D222" s="29" t="n"/>
+      <c r="E222" s="29" t="n"/>
+      <c r="F222" s="29" t="n"/>
+      <c r="G222" s="29" t="n"/>
+      <c r="H222" s="29" t="n"/>
+      <c r="I222" s="29" t="n"/>
+      <c r="J222" s="29" t="n"/>
+      <c r="K222" s="29">
+        <f>SUM(J223:J224)*PARAMETROS!$B$16</f>
+        <v/>
+      </c>
+      <c r="L222" s="28" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="30" t="n"/>
       <c r="B223" s="30" t="inlineStr">
         <is>
-          <t>Caja de caida CC</t>
+          <t>Excavacion de zanjas y cajas</t>
         </is>
       </c>
       <c r="C223" s="31" t="n">
@@ -16042,143 +15842,137 @@
       <c r="H223" s="31" t="n"/>
       <c r="I223" s="31" t="n"/>
       <c r="J223" s="31">
-        <f>'COLECTOR TRAMOS'!N35</f>
+        <f>K185</f>
         <v/>
       </c>
       <c r="K223" s="31" t="n"/>
       <c r="L223" s="30" t="n"/>
     </row>
     <row r="224">
-      <c r="A224" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.02.04</t>
-        </is>
-      </c>
-      <c r="B224" s="28" t="inlineStr">
-        <is>
-          <t>ELIMINACIÓN DE MATERIAL EXCEDENTE</t>
-        </is>
-      </c>
-      <c r="C224" s="29" t="n"/>
-      <c r="D224" s="29" t="n"/>
-      <c r="E224" s="29" t="n"/>
-      <c r="F224" s="29" t="n"/>
-      <c r="G224" s="29" t="n"/>
-      <c r="H224" s="29" t="n"/>
-      <c r="I224" s="29" t="n"/>
-      <c r="J224" s="29" t="n"/>
-      <c r="K224" s="29">
-        <f>SUM(J225:J226)*PARAMETROS!$B$16</f>
-        <v/>
-      </c>
-      <c r="L224" s="28" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
+      <c r="A224" s="30" t="n"/>
+      <c r="B224" s="30" t="inlineStr">
+        <is>
+          <t>Relleno compactado (se descuenta)</t>
+        </is>
+      </c>
+      <c r="C224" s="31" t="n">
+        <v>-1</v>
+      </c>
+      <c r="D224" s="31" t="n"/>
+      <c r="E224" s="31" t="n"/>
+      <c r="F224" s="31" t="n"/>
+      <c r="G224" s="31" t="n"/>
+      <c r="H224" s="31" t="n"/>
+      <c r="I224" s="31" t="n"/>
+      <c r="J224" s="31">
+        <f>-K205</f>
+        <v/>
+      </c>
+      <c r="K224" s="31" t="n"/>
+      <c r="L224" s="30" t="n"/>
     </row>
     <row r="225">
-      <c r="A225" s="30" t="n"/>
-      <c r="B225" s="30" t="inlineStr">
-        <is>
-          <t>Excavacion de zanjas y cajas</t>
-        </is>
-      </c>
-      <c r="C225" s="31" t="n">
+      <c r="A225" s="217" t="inlineStr">
+        <is>
+          <t>01.04.04.03</t>
+        </is>
+      </c>
+      <c r="B225" s="217" t="inlineStr">
+        <is>
+          <t>OBRAS DE CONCRETO SIMPLE</t>
+        </is>
+      </c>
+      <c r="C225" s="313" t="n"/>
+      <c r="D225" s="313" t="n"/>
+      <c r="E225" s="313" t="n"/>
+      <c r="F225" s="313" t="n"/>
+      <c r="G225" s="313" t="n"/>
+      <c r="H225" s="313" t="n"/>
+      <c r="I225" s="313" t="n"/>
+      <c r="J225" s="313" t="n"/>
+      <c r="K225" s="313" t="n"/>
+      <c r="L225" s="314" t="n"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.03.01</t>
+        </is>
+      </c>
+      <c r="B226" s="28" t="inlineStr">
+        <is>
+          <t>CONCRETO f'c=100 kg/cm2 PARA SOLADO E=2" (0.05 m)</t>
+        </is>
+      </c>
+      <c r="C226" s="29" t="n"/>
+      <c r="D226" s="29" t="n"/>
+      <c r="E226" s="29" t="n"/>
+      <c r="F226" s="29" t="n"/>
+      <c r="G226" s="29" t="n"/>
+      <c r="H226" s="29" t="n"/>
+      <c r="I226" s="29" t="n"/>
+      <c r="J226" s="29" t="n"/>
+      <c r="K226" s="29">
+        <f>SUM(J227:J235)</f>
+        <v/>
+      </c>
+      <c r="L226" s="28" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="30" t="n"/>
+      <c r="B227" s="30" t="inlineStr">
+        <is>
+          <t>Tramo normal (0+000.00 - 0+026.32)</t>
+        </is>
+      </c>
+      <c r="C227" s="31" t="n">
         <v>1</v>
       </c>
-      <c r="D225" s="31" t="n"/>
-      <c r="E225" s="31" t="n"/>
-      <c r="F225" s="31" t="n"/>
-      <c r="G225" s="31" t="n"/>
-      <c r="H225" s="31" t="n"/>
-      <c r="I225" s="31" t="n"/>
-      <c r="J225" s="31">
-        <f>K185</f>
-        <v/>
-      </c>
-      <c r="K225" s="31" t="n"/>
-      <c r="L225" s="30" t="n"/>
-    </row>
-    <row r="226">
-      <c r="A226" s="30" t="n"/>
-      <c r="B226" s="30" t="inlineStr">
-        <is>
-          <t>Relleno compactado (se descuenta)</t>
-        </is>
-      </c>
-      <c r="C226" s="31" t="n">
-        <v>-1</v>
-      </c>
-      <c r="D226" s="31" t="n"/>
-      <c r="E226" s="31" t="n"/>
-      <c r="F226" s="31" t="n"/>
-      <c r="G226" s="31" t="n"/>
-      <c r="H226" s="31" t="n"/>
-      <c r="I226" s="31" t="n"/>
-      <c r="J226" s="31">
-        <f>-K207</f>
-        <v/>
-      </c>
-      <c r="K226" s="31" t="n"/>
-      <c r="L226" s="30" t="n"/>
-    </row>
-    <row r="227">
-      <c r="A227" s="217" t="inlineStr">
-        <is>
-          <t>01.04.04.03</t>
-        </is>
-      </c>
-      <c r="B227" s="217" t="inlineStr">
-        <is>
-          <t>OBRAS DE CONCRETO SIMPLE</t>
-        </is>
-      </c>
-      <c r="C227" s="313" t="n"/>
-      <c r="D227" s="313" t="n"/>
-      <c r="E227" s="313" t="n"/>
-      <c r="F227" s="313" t="n"/>
-      <c r="G227" s="313" t="n"/>
-      <c r="H227" s="313" t="n"/>
-      <c r="I227" s="313" t="n"/>
-      <c r="J227" s="313" t="n"/>
-      <c r="K227" s="313" t="n"/>
-      <c r="L227" s="314" t="n"/>
+      <c r="D227" s="31" t="n"/>
+      <c r="E227" s="31" t="n"/>
+      <c r="F227" s="31" t="n"/>
+      <c r="G227" s="31" t="n"/>
+      <c r="H227" s="31" t="n"/>
+      <c r="I227" s="31" t="n"/>
+      <c r="J227" s="31">
+        <f>'COLECTOR TRAMOS'!Q22</f>
+        <v/>
+      </c>
+      <c r="K227" s="31" t="n"/>
+      <c r="L227" s="30" t="n"/>
     </row>
     <row r="228">
-      <c r="A228" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.03.01</t>
-        </is>
-      </c>
-      <c r="B228" s="28" t="inlineStr">
-        <is>
-          <t>CONCRETO f'c=100 kg/cm2 PARA SOLADO E=2" (0.05 m)</t>
-        </is>
-      </c>
-      <c r="C228" s="29" t="n"/>
-      <c r="D228" s="29" t="n"/>
-      <c r="E228" s="29" t="n"/>
-      <c r="F228" s="29" t="n"/>
-      <c r="G228" s="29" t="n"/>
-      <c r="H228" s="29" t="n"/>
-      <c r="I228" s="29" t="n"/>
-      <c r="J228" s="29" t="n"/>
-      <c r="K228" s="29">
-        <f>SUM(J229:J239)</f>
-        <v/>
-      </c>
-      <c r="L228" s="28" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
+      <c r="A228" s="30" t="n"/>
+      <c r="B228" s="30" t="inlineStr">
+        <is>
+          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
+        </is>
+      </c>
+      <c r="C228" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D228" s="31" t="n"/>
+      <c r="E228" s="31" t="n"/>
+      <c r="F228" s="31" t="n"/>
+      <c r="G228" s="31" t="n"/>
+      <c r="H228" s="31" t="n"/>
+      <c r="I228" s="31" t="n"/>
+      <c r="J228" s="31">
+        <f>'COLECTOR TRAMOS'!Q23</f>
+        <v/>
+      </c>
+      <c r="K228" s="31" t="n"/>
+      <c r="L228" s="30" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="30" t="n"/>
       <c r="B229" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+000.00 - 0+026.32)</t>
+          <t>Tramo normal (0+031.33 - 0+039.04)</t>
         </is>
       </c>
       <c r="C229" s="31" t="n">
@@ -16191,7 +15985,7 @@
       <c r="H229" s="31" t="n"/>
       <c r="I229" s="31" t="n"/>
       <c r="J229" s="31">
-        <f>'COLECTOR TRAMOS'!Q22</f>
+        <f>'COLECTOR TRAMOS'!Q24</f>
         <v/>
       </c>
       <c r="K229" s="31" t="n"/>
@@ -16201,7 +15995,7 @@
       <c r="A230" s="30" t="n"/>
       <c r="B230" s="30" t="inlineStr">
         <is>
-          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
+          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
         </is>
       </c>
       <c r="C230" s="31" t="n">
@@ -16214,7 +16008,7 @@
       <c r="H230" s="31" t="n"/>
       <c r="I230" s="31" t="n"/>
       <c r="J230" s="31">
-        <f>'COLECTOR TRAMOS'!Q23</f>
+        <f>'COLECTOR TRAMOS'!Q25</f>
         <v/>
       </c>
       <c r="K230" s="31" t="n"/>
@@ -16224,7 +16018,7 @@
       <c r="A231" s="30" t="n"/>
       <c r="B231" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+031.33 - 0+039.04)</t>
+          <t>Tramo normal (0+041.04 - 0+058.81)</t>
         </is>
       </c>
       <c r="C231" s="31" t="n">
@@ -16237,7 +16031,7 @@
       <c r="H231" s="31" t="n"/>
       <c r="I231" s="31" t="n"/>
       <c r="J231" s="31">
-        <f>'COLECTOR TRAMOS'!Q24</f>
+        <f>'COLECTOR TRAMOS'!Q26</f>
         <v/>
       </c>
       <c r="K231" s="31" t="n"/>
@@ -16247,7 +16041,7 @@
       <c r="A232" s="30" t="n"/>
       <c r="B232" s="30" t="inlineStr">
         <is>
-          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
+          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
         </is>
       </c>
       <c r="C232" s="31" t="n">
@@ -16260,7 +16054,7 @@
       <c r="H232" s="31" t="n"/>
       <c r="I232" s="31" t="n"/>
       <c r="J232" s="31">
-        <f>'COLECTOR TRAMOS'!Q25</f>
+        <f>'COLECTOR TRAMOS'!Q27</f>
         <v/>
       </c>
       <c r="K232" s="31" t="n"/>
@@ -16270,7 +16064,7 @@
       <c r="A233" s="30" t="n"/>
       <c r="B233" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+041.04 - 0+058.81)</t>
+          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
         </is>
       </c>
       <c r="C233" s="31" t="n">
@@ -16283,7 +16077,7 @@
       <c r="H233" s="31" t="n"/>
       <c r="I233" s="31" t="n"/>
       <c r="J233" s="31">
-        <f>'COLECTOR TRAMOS'!Q26</f>
+        <f>'COLECTOR TRAMOS'!Q28</f>
         <v/>
       </c>
       <c r="K233" s="31" t="n"/>
@@ -16293,7 +16087,7 @@
       <c r="A234" s="30" t="n"/>
       <c r="B234" s="30" t="inlineStr">
         <is>
-          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
+          <t>Caja de llegada CL</t>
         </is>
       </c>
       <c r="C234" s="31" t="n">
@@ -16306,7 +16100,7 @@
       <c r="H234" s="31" t="n"/>
       <c r="I234" s="31" t="n"/>
       <c r="J234" s="31">
-        <f>'COLECTOR TRAMOS'!Q27</f>
+        <f>'COLECTOR TRAMOS'!G34</f>
         <v/>
       </c>
       <c r="K234" s="31" t="n"/>
@@ -16316,7 +16110,7 @@
       <c r="A235" s="30" t="n"/>
       <c r="B235" s="30" t="inlineStr">
         <is>
-          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
+          <t>Caja de caida CC</t>
         </is>
       </c>
       <c r="C235" s="31" t="n">
@@ -16329,63 +16123,68 @@
       <c r="H235" s="31" t="n"/>
       <c r="I235" s="31" t="n"/>
       <c r="J235" s="31">
-        <f>'COLECTOR TRAMOS'!Q28</f>
+        <f>'COLECTOR TRAMOS'!G35</f>
         <v/>
       </c>
       <c r="K235" s="31" t="n"/>
       <c r="L235" s="30" t="n"/>
     </row>
     <row r="236">
-      <c r="A236" s="30" t="n"/>
-      <c r="B236" s="30" t="inlineStr">
-        <is>
-          <t>Caja de llegada CL</t>
-        </is>
-      </c>
-      <c r="C236" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D236" s="31" t="n"/>
-      <c r="E236" s="31" t="n"/>
-      <c r="F236" s="31" t="n"/>
-      <c r="G236" s="31" t="n"/>
-      <c r="H236" s="31" t="n"/>
-      <c r="I236" s="31" t="n"/>
-      <c r="J236" s="31">
-        <f>'COLECTOR TRAMOS'!G34</f>
-        <v/>
-      </c>
-      <c r="K236" s="31" t="n"/>
-      <c r="L236" s="30" t="n"/>
+      <c r="A236" s="217" t="inlineStr">
+        <is>
+          <t>01.04.04.04</t>
+        </is>
+      </c>
+      <c r="B236" s="217" t="inlineStr">
+        <is>
+          <t>OBRAS DE CONCRETO ARMADO - COLECTOR Y CAJAS</t>
+        </is>
+      </c>
+      <c r="C236" s="313" t="n"/>
+      <c r="D236" s="313" t="n"/>
+      <c r="E236" s="313" t="n"/>
+      <c r="F236" s="313" t="n"/>
+      <c r="G236" s="313" t="n"/>
+      <c r="H236" s="313" t="n"/>
+      <c r="I236" s="313" t="n"/>
+      <c r="J236" s="313" t="n"/>
+      <c r="K236" s="313" t="n"/>
+      <c r="L236" s="314" t="n"/>
     </row>
     <row r="237">
-      <c r="A237" s="30" t="n"/>
-      <c r="B237" s="30" t="inlineStr">
-        <is>
-          <t>Caja de caida CC</t>
-        </is>
-      </c>
-      <c r="C237" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D237" s="31" t="n"/>
-      <c r="E237" s="31" t="n"/>
-      <c r="F237" s="31" t="n"/>
-      <c r="G237" s="31" t="n"/>
-      <c r="H237" s="31" t="n"/>
-      <c r="I237" s="31" t="n"/>
-      <c r="J237" s="31">
-        <f>'COLECTOR TRAMOS'!G35</f>
-        <v/>
-      </c>
-      <c r="K237" s="31" t="n"/>
-      <c r="L237" s="30" t="n"/>
+      <c r="A237" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.04.01</t>
+        </is>
+      </c>
+      <c r="B237" s="28" t="inlineStr">
+        <is>
+          <t>CONCRETO f'c=210 kg/cm2 EN LOSA DE FONDO</t>
+        </is>
+      </c>
+      <c r="C237" s="29" t="n"/>
+      <c r="D237" s="29" t="n"/>
+      <c r="E237" s="29" t="n"/>
+      <c r="F237" s="29" t="n"/>
+      <c r="G237" s="29" t="n"/>
+      <c r="H237" s="29" t="n"/>
+      <c r="I237" s="29" t="n"/>
+      <c r="J237" s="29" t="n"/>
+      <c r="K237" s="29">
+        <f>SUM(J238:J246)</f>
+        <v/>
+      </c>
+      <c r="L237" s="28" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="30" t="n"/>
       <c r="B238" s="30" t="inlineStr">
         <is>
-          <t>Prolongacion cuneta Eje 11</t>
+          <t>Tramo normal (0+000.00 - 0+026.32)</t>
         </is>
       </c>
       <c r="C238" s="31" t="n">
@@ -16398,7 +16197,7 @@
       <c r="H238" s="31" t="n"/>
       <c r="I238" s="31" t="n"/>
       <c r="J238" s="31">
-        <f>'COLECTOR TRAMOS'!G36</f>
+        <f>'COLECTOR TRAMOS'!R22</f>
         <v/>
       </c>
       <c r="K238" s="31" t="n"/>
@@ -16408,7 +16207,7 @@
       <c r="A239" s="30" t="n"/>
       <c r="B239" s="30" t="inlineStr">
         <is>
-          <t>Prolongacion cuneta Eje 12</t>
+          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
         </is>
       </c>
       <c r="C239" s="31" t="n">
@@ -16421,68 +16220,63 @@
       <c r="H239" s="31" t="n"/>
       <c r="I239" s="31" t="n"/>
       <c r="J239" s="31">
-        <f>'COLECTOR TRAMOS'!G37</f>
+        <f>'COLECTOR TRAMOS'!R23</f>
         <v/>
       </c>
       <c r="K239" s="31" t="n"/>
       <c r="L239" s="30" t="n"/>
     </row>
     <row r="240">
-      <c r="A240" s="217" t="inlineStr">
-        <is>
-          <t>01.04.04.04</t>
-        </is>
-      </c>
-      <c r="B240" s="217" t="inlineStr">
-        <is>
-          <t>OBRAS DE CONCRETO ARMADO - COLECTOR Y CAJAS</t>
-        </is>
-      </c>
-      <c r="C240" s="313" t="n"/>
-      <c r="D240" s="313" t="n"/>
-      <c r="E240" s="313" t="n"/>
-      <c r="F240" s="313" t="n"/>
-      <c r="G240" s="313" t="n"/>
-      <c r="H240" s="313" t="n"/>
-      <c r="I240" s="313" t="n"/>
-      <c r="J240" s="313" t="n"/>
-      <c r="K240" s="313" t="n"/>
-      <c r="L240" s="314" t="n"/>
+      <c r="A240" s="30" t="n"/>
+      <c r="B240" s="30" t="inlineStr">
+        <is>
+          <t>Tramo normal (0+031.33 - 0+039.04)</t>
+        </is>
+      </c>
+      <c r="C240" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D240" s="31" t="n"/>
+      <c r="E240" s="31" t="n"/>
+      <c r="F240" s="31" t="n"/>
+      <c r="G240" s="31" t="n"/>
+      <c r="H240" s="31" t="n"/>
+      <c r="I240" s="31" t="n"/>
+      <c r="J240" s="31">
+        <f>'COLECTOR TRAMOS'!R24</f>
+        <v/>
+      </c>
+      <c r="K240" s="31" t="n"/>
+      <c r="L240" s="30" t="n"/>
     </row>
     <row r="241">
-      <c r="A241" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.04.01</t>
-        </is>
-      </c>
-      <c r="B241" s="28" t="inlineStr">
-        <is>
-          <t>CONCRETO f'c=210 kg/cm2 EN LOSA DE FONDO</t>
-        </is>
-      </c>
-      <c r="C241" s="29" t="n"/>
-      <c r="D241" s="29" t="n"/>
-      <c r="E241" s="29" t="n"/>
-      <c r="F241" s="29" t="n"/>
-      <c r="G241" s="29" t="n"/>
-      <c r="H241" s="29" t="n"/>
-      <c r="I241" s="29" t="n"/>
-      <c r="J241" s="29" t="n"/>
-      <c r="K241" s="29">
-        <f>SUM(J242:J250)</f>
-        <v/>
-      </c>
-      <c r="L241" s="28" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
+      <c r="A241" s="30" t="n"/>
+      <c r="B241" s="30" t="inlineStr">
+        <is>
+          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
+        </is>
+      </c>
+      <c r="C241" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D241" s="31" t="n"/>
+      <c r="E241" s="31" t="n"/>
+      <c r="F241" s="31" t="n"/>
+      <c r="G241" s="31" t="n"/>
+      <c r="H241" s="31" t="n"/>
+      <c r="I241" s="31" t="n"/>
+      <c r="J241" s="31">
+        <f>'COLECTOR TRAMOS'!R25</f>
+        <v/>
+      </c>
+      <c r="K241" s="31" t="n"/>
+      <c r="L241" s="30" t="n"/>
     </row>
     <row r="242">
       <c r="A242" s="30" t="n"/>
       <c r="B242" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+000.00 - 0+026.32)</t>
+          <t>Tramo normal (0+041.04 - 0+058.81)</t>
         </is>
       </c>
       <c r="C242" s="31" t="n">
@@ -16495,7 +16289,7 @@
       <c r="H242" s="31" t="n"/>
       <c r="I242" s="31" t="n"/>
       <c r="J242" s="31">
-        <f>'COLECTOR TRAMOS'!R22</f>
+        <f>'COLECTOR TRAMOS'!R26</f>
         <v/>
       </c>
       <c r="K242" s="31" t="n"/>
@@ -16505,7 +16299,7 @@
       <c r="A243" s="30" t="n"/>
       <c r="B243" s="30" t="inlineStr">
         <is>
-          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
+          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
         </is>
       </c>
       <c r="C243" s="31" t="n">
@@ -16518,7 +16312,7 @@
       <c r="H243" s="31" t="n"/>
       <c r="I243" s="31" t="n"/>
       <c r="J243" s="31">
-        <f>'COLECTOR TRAMOS'!R23</f>
+        <f>'COLECTOR TRAMOS'!R27</f>
         <v/>
       </c>
       <c r="K243" s="31" t="n"/>
@@ -16528,7 +16322,7 @@
       <c r="A244" s="30" t="n"/>
       <c r="B244" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+031.33 - 0+039.04)</t>
+          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
         </is>
       </c>
       <c r="C244" s="31" t="n">
@@ -16541,7 +16335,7 @@
       <c r="H244" s="31" t="n"/>
       <c r="I244" s="31" t="n"/>
       <c r="J244" s="31">
-        <f>'COLECTOR TRAMOS'!R24</f>
+        <f>'COLECTOR TRAMOS'!R28</f>
         <v/>
       </c>
       <c r="K244" s="31" t="n"/>
@@ -16551,7 +16345,7 @@
       <c r="A245" s="30" t="n"/>
       <c r="B245" s="30" t="inlineStr">
         <is>
-          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
+          <t>Caja de llegada CL</t>
         </is>
       </c>
       <c r="C245" s="31" t="n">
@@ -16564,7 +16358,7 @@
       <c r="H245" s="31" t="n"/>
       <c r="I245" s="31" t="n"/>
       <c r="J245" s="31">
-        <f>'COLECTOR TRAMOS'!R25</f>
+        <f>'COLECTOR TRAMOS'!H34</f>
         <v/>
       </c>
       <c r="K245" s="31" t="n"/>
@@ -16574,7 +16368,7 @@
       <c r="A246" s="30" t="n"/>
       <c r="B246" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+041.04 - 0+058.81)</t>
+          <t>Caja de caida CC (incluye umbral)</t>
         </is>
       </c>
       <c r="C246" s="31" t="n">
@@ -16587,40 +16381,46 @@
       <c r="H246" s="31" t="n"/>
       <c r="I246" s="31" t="n"/>
       <c r="J246" s="31">
-        <f>'COLECTOR TRAMOS'!R26</f>
+        <f>'COLECTOR TRAMOS'!H35</f>
         <v/>
       </c>
       <c r="K246" s="31" t="n"/>
       <c r="L246" s="30" t="n"/>
     </row>
     <row r="247">
-      <c r="A247" s="30" t="n"/>
-      <c r="B247" s="30" t="inlineStr">
-        <is>
-          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
-        </is>
-      </c>
-      <c r="C247" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D247" s="31" t="n"/>
-      <c r="E247" s="31" t="n"/>
-      <c r="F247" s="31" t="n"/>
-      <c r="G247" s="31" t="n"/>
-      <c r="H247" s="31" t="n"/>
-      <c r="I247" s="31" t="n"/>
-      <c r="J247" s="31">
-        <f>'COLECTOR TRAMOS'!R27</f>
-        <v/>
-      </c>
-      <c r="K247" s="31" t="n"/>
-      <c r="L247" s="30" t="n"/>
+      <c r="A247" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.04.02</t>
+        </is>
+      </c>
+      <c r="B247" s="28" t="inlineStr">
+        <is>
+          <t>CONCRETO f'c=210 kg/cm2 EN MUROS</t>
+        </is>
+      </c>
+      <c r="C247" s="29" t="n"/>
+      <c r="D247" s="29" t="n"/>
+      <c r="E247" s="29" t="n"/>
+      <c r="F247" s="29" t="n"/>
+      <c r="G247" s="29" t="n"/>
+      <c r="H247" s="29" t="n"/>
+      <c r="I247" s="29" t="n"/>
+      <c r="J247" s="29" t="n"/>
+      <c r="K247" s="29">
+        <f>SUM(J248:J256)</f>
+        <v/>
+      </c>
+      <c r="L247" s="28" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="30" t="n"/>
       <c r="B248" s="30" t="inlineStr">
         <is>
-          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
+          <t>Tramo normal (0+000.00 - 0+026.32)</t>
         </is>
       </c>
       <c r="C248" s="31" t="n">
@@ -16633,7 +16433,7 @@
       <c r="H248" s="31" t="n"/>
       <c r="I248" s="31" t="n"/>
       <c r="J248" s="31">
-        <f>'COLECTOR TRAMOS'!R28</f>
+        <f>'COLECTOR TRAMOS'!S22</f>
         <v/>
       </c>
       <c r="K248" s="31" t="n"/>
@@ -16643,7 +16443,7 @@
       <c r="A249" s="30" t="n"/>
       <c r="B249" s="30" t="inlineStr">
         <is>
-          <t>Caja de llegada CL</t>
+          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
         </is>
       </c>
       <c r="C249" s="31" t="n">
@@ -16656,7 +16456,7 @@
       <c r="H249" s="31" t="n"/>
       <c r="I249" s="31" t="n"/>
       <c r="J249" s="31">
-        <f>'COLECTOR TRAMOS'!H34</f>
+        <f>'COLECTOR TRAMOS'!S23</f>
         <v/>
       </c>
       <c r="K249" s="31" t="n"/>
@@ -16666,7 +16466,7 @@
       <c r="A250" s="30" t="n"/>
       <c r="B250" s="30" t="inlineStr">
         <is>
-          <t>Caja de caida CC (incluye umbral)</t>
+          <t>Tramo normal (0+031.33 - 0+039.04)</t>
         </is>
       </c>
       <c r="C250" s="31" t="n">
@@ -16679,46 +16479,40 @@
       <c r="H250" s="31" t="n"/>
       <c r="I250" s="31" t="n"/>
       <c r="J250" s="31">
-        <f>'COLECTOR TRAMOS'!H35</f>
+        <f>'COLECTOR TRAMOS'!S24</f>
         <v/>
       </c>
       <c r="K250" s="31" t="n"/>
       <c r="L250" s="30" t="n"/>
     </row>
     <row r="251">
-      <c r="A251" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.04.02</t>
-        </is>
-      </c>
-      <c r="B251" s="28" t="inlineStr">
-        <is>
-          <t>CONCRETO f'c=210 kg/cm2 EN MUROS</t>
-        </is>
-      </c>
-      <c r="C251" s="29" t="n"/>
-      <c r="D251" s="29" t="n"/>
-      <c r="E251" s="29" t="n"/>
-      <c r="F251" s="29" t="n"/>
-      <c r="G251" s="29" t="n"/>
-      <c r="H251" s="29" t="n"/>
-      <c r="I251" s="29" t="n"/>
-      <c r="J251" s="29" t="n"/>
-      <c r="K251" s="29">
-        <f>SUM(J252:J260)</f>
-        <v/>
-      </c>
-      <c r="L251" s="28" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
+      <c r="A251" s="30" t="n"/>
+      <c r="B251" s="30" t="inlineStr">
+        <is>
+          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
+        </is>
+      </c>
+      <c r="C251" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D251" s="31" t="n"/>
+      <c r="E251" s="31" t="n"/>
+      <c r="F251" s="31" t="n"/>
+      <c r="G251" s="31" t="n"/>
+      <c r="H251" s="31" t="n"/>
+      <c r="I251" s="31" t="n"/>
+      <c r="J251" s="31">
+        <f>'COLECTOR TRAMOS'!S25</f>
+        <v/>
+      </c>
+      <c r="K251" s="31" t="n"/>
+      <c r="L251" s="30" t="n"/>
     </row>
     <row r="252">
       <c r="A252" s="30" t="n"/>
       <c r="B252" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+000.00 - 0+026.32)</t>
+          <t>Tramo normal (0+041.04 - 0+058.81)</t>
         </is>
       </c>
       <c r="C252" s="31" t="n">
@@ -16731,7 +16525,7 @@
       <c r="H252" s="31" t="n"/>
       <c r="I252" s="31" t="n"/>
       <c r="J252" s="31">
-        <f>'COLECTOR TRAMOS'!S22</f>
+        <f>'COLECTOR TRAMOS'!S26</f>
         <v/>
       </c>
       <c r="K252" s="31" t="n"/>
@@ -16741,7 +16535,7 @@
       <c r="A253" s="30" t="n"/>
       <c r="B253" s="30" t="inlineStr">
         <is>
-          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
+          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
         </is>
       </c>
       <c r="C253" s="31" t="n">
@@ -16754,7 +16548,7 @@
       <c r="H253" s="31" t="n"/>
       <c r="I253" s="31" t="n"/>
       <c r="J253" s="31">
-        <f>'COLECTOR TRAMOS'!S23</f>
+        <f>'COLECTOR TRAMOS'!S27</f>
         <v/>
       </c>
       <c r="K253" s="31" t="n"/>
@@ -16764,7 +16558,7 @@
       <c r="A254" s="30" t="n"/>
       <c r="B254" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+031.33 - 0+039.04)</t>
+          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
         </is>
       </c>
       <c r="C254" s="31" t="n">
@@ -16777,7 +16571,7 @@
       <c r="H254" s="31" t="n"/>
       <c r="I254" s="31" t="n"/>
       <c r="J254" s="31">
-        <f>'COLECTOR TRAMOS'!S24</f>
+        <f>'COLECTOR TRAMOS'!S28</f>
         <v/>
       </c>
       <c r="K254" s="31" t="n"/>
@@ -16787,7 +16581,7 @@
       <c r="A255" s="30" t="n"/>
       <c r="B255" s="30" t="inlineStr">
         <is>
-          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
+          <t>Caja de llegada CL</t>
         </is>
       </c>
       <c r="C255" s="31" t="n">
@@ -16800,7 +16594,7 @@
       <c r="H255" s="31" t="n"/>
       <c r="I255" s="31" t="n"/>
       <c r="J255" s="31">
-        <f>'COLECTOR TRAMOS'!S25</f>
+        <f>'COLECTOR TRAMOS'!I34</f>
         <v/>
       </c>
       <c r="K255" s="31" t="n"/>
@@ -16810,7 +16604,7 @@
       <c r="A256" s="30" t="n"/>
       <c r="B256" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+041.04 - 0+058.81)</t>
+          <t>Caja de caida CC</t>
         </is>
       </c>
       <c r="C256" s="31" t="n">
@@ -16823,40 +16617,46 @@
       <c r="H256" s="31" t="n"/>
       <c r="I256" s="31" t="n"/>
       <c r="J256" s="31">
-        <f>'COLECTOR TRAMOS'!S26</f>
+        <f>'COLECTOR TRAMOS'!I35</f>
         <v/>
       </c>
       <c r="K256" s="31" t="n"/>
       <c r="L256" s="30" t="n"/>
     </row>
     <row r="257">
-      <c r="A257" s="30" t="n"/>
-      <c r="B257" s="30" t="inlineStr">
-        <is>
-          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
-        </is>
-      </c>
-      <c r="C257" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D257" s="31" t="n"/>
-      <c r="E257" s="31" t="n"/>
-      <c r="F257" s="31" t="n"/>
-      <c r="G257" s="31" t="n"/>
-      <c r="H257" s="31" t="n"/>
-      <c r="I257" s="31" t="n"/>
-      <c r="J257" s="31">
-        <f>'COLECTOR TRAMOS'!S27</f>
-        <v/>
-      </c>
-      <c r="K257" s="31" t="n"/>
-      <c r="L257" s="30" t="n"/>
+      <c r="A257" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.04.03</t>
+        </is>
+      </c>
+      <c r="B257" s="28" t="inlineStr">
+        <is>
+          <t>CONCRETO f'c=210 kg/cm2 EN LOSA SUPERIOR (incluye bordes de registro)</t>
+        </is>
+      </c>
+      <c r="C257" s="29" t="n"/>
+      <c r="D257" s="29" t="n"/>
+      <c r="E257" s="29" t="n"/>
+      <c r="F257" s="29" t="n"/>
+      <c r="G257" s="29" t="n"/>
+      <c r="H257" s="29" t="n"/>
+      <c r="I257" s="29" t="n"/>
+      <c r="J257" s="29" t="n"/>
+      <c r="K257" s="29">
+        <f>SUM(J258:J268)</f>
+        <v/>
+      </c>
+      <c r="L257" s="28" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="30" t="n"/>
       <c r="B258" s="30" t="inlineStr">
         <is>
-          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
+          <t>Tramo normal (0+000.00 - 0+026.32)</t>
         </is>
       </c>
       <c r="C258" s="31" t="n">
@@ -16869,7 +16669,7 @@
       <c r="H258" s="31" t="n"/>
       <c r="I258" s="31" t="n"/>
       <c r="J258" s="31">
-        <f>'COLECTOR TRAMOS'!S28</f>
+        <f>'COLECTOR TRAMOS'!T22</f>
         <v/>
       </c>
       <c r="K258" s="31" t="n"/>
@@ -16879,7 +16679,7 @@
       <c r="A259" s="30" t="n"/>
       <c r="B259" s="30" t="inlineStr">
         <is>
-          <t>Caja de llegada CL</t>
+          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
         </is>
       </c>
       <c r="C259" s="31" t="n">
@@ -16892,7 +16692,7 @@
       <c r="H259" s="31" t="n"/>
       <c r="I259" s="31" t="n"/>
       <c r="J259" s="31">
-        <f>'COLECTOR TRAMOS'!I34</f>
+        <f>'COLECTOR TRAMOS'!T23</f>
         <v/>
       </c>
       <c r="K259" s="31" t="n"/>
@@ -16902,7 +16702,7 @@
       <c r="A260" s="30" t="n"/>
       <c r="B260" s="30" t="inlineStr">
         <is>
-          <t>Caja de caida CC</t>
+          <t>Tramo normal (0+031.33 - 0+039.04)</t>
         </is>
       </c>
       <c r="C260" s="31" t="n">
@@ -16915,46 +16715,40 @@
       <c r="H260" s="31" t="n"/>
       <c r="I260" s="31" t="n"/>
       <c r="J260" s="31">
-        <f>'COLECTOR TRAMOS'!I35</f>
+        <f>'COLECTOR TRAMOS'!T24</f>
         <v/>
       </c>
       <c r="K260" s="31" t="n"/>
       <c r="L260" s="30" t="n"/>
     </row>
     <row r="261">
-      <c r="A261" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.04.03</t>
-        </is>
-      </c>
-      <c r="B261" s="28" t="inlineStr">
-        <is>
-          <t>CONCRETO f'c=210 kg/cm2 EN LOSA SUPERIOR (incluye bordes de registro)</t>
-        </is>
-      </c>
-      <c r="C261" s="29" t="n"/>
-      <c r="D261" s="29" t="n"/>
-      <c r="E261" s="29" t="n"/>
-      <c r="F261" s="29" t="n"/>
-      <c r="G261" s="29" t="n"/>
-      <c r="H261" s="29" t="n"/>
-      <c r="I261" s="29" t="n"/>
-      <c r="J261" s="29" t="n"/>
-      <c r="K261" s="29">
-        <f>SUM(J262:J272)</f>
-        <v/>
-      </c>
-      <c r="L261" s="28" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
+      <c r="A261" s="30" t="n"/>
+      <c r="B261" s="30" t="inlineStr">
+        <is>
+          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
+        </is>
+      </c>
+      <c r="C261" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D261" s="31" t="n"/>
+      <c r="E261" s="31" t="n"/>
+      <c r="F261" s="31" t="n"/>
+      <c r="G261" s="31" t="n"/>
+      <c r="H261" s="31" t="n"/>
+      <c r="I261" s="31" t="n"/>
+      <c r="J261" s="31">
+        <f>'COLECTOR TRAMOS'!T25</f>
+        <v/>
+      </c>
+      <c r="K261" s="31" t="n"/>
+      <c r="L261" s="30" t="n"/>
     </row>
     <row r="262">
       <c r="A262" s="30" t="n"/>
       <c r="B262" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+000.00 - 0+026.32)</t>
+          <t>Tramo normal (0+041.04 - 0+058.81)</t>
         </is>
       </c>
       <c r="C262" s="31" t="n">
@@ -16967,7 +16761,7 @@
       <c r="H262" s="31" t="n"/>
       <c r="I262" s="31" t="n"/>
       <c r="J262" s="31">
-        <f>'COLECTOR TRAMOS'!T22</f>
+        <f>'COLECTOR TRAMOS'!T26</f>
         <v/>
       </c>
       <c r="K262" s="31" t="n"/>
@@ -16977,7 +16771,7 @@
       <c r="A263" s="30" t="n"/>
       <c r="B263" s="30" t="inlineStr">
         <is>
-          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
+          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
         </is>
       </c>
       <c r="C263" s="31" t="n">
@@ -16990,7 +16784,7 @@
       <c r="H263" s="31" t="n"/>
       <c r="I263" s="31" t="n"/>
       <c r="J263" s="31">
-        <f>'COLECTOR TRAMOS'!T23</f>
+        <f>'COLECTOR TRAMOS'!T27</f>
         <v/>
       </c>
       <c r="K263" s="31" t="n"/>
@@ -17000,7 +16794,7 @@
       <c r="A264" s="30" t="n"/>
       <c r="B264" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+031.33 - 0+039.04)</t>
+          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
         </is>
       </c>
       <c r="C264" s="31" t="n">
@@ -17013,7 +16807,7 @@
       <c r="H264" s="31" t="n"/>
       <c r="I264" s="31" t="n"/>
       <c r="J264" s="31">
-        <f>'COLECTOR TRAMOS'!T24</f>
+        <f>'COLECTOR TRAMOS'!T28</f>
         <v/>
       </c>
       <c r="K264" s="31" t="n"/>
@@ -17023,7 +16817,7 @@
       <c r="A265" s="30" t="n"/>
       <c r="B265" s="30" t="inlineStr">
         <is>
-          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
+          <t>Caja de llegada CL</t>
         </is>
       </c>
       <c r="C265" s="31" t="n">
@@ -17036,7 +16830,7 @@
       <c r="H265" s="31" t="n"/>
       <c r="I265" s="31" t="n"/>
       <c r="J265" s="31">
-        <f>'COLECTOR TRAMOS'!T25</f>
+        <f>'COLECTOR TRAMOS'!J34</f>
         <v/>
       </c>
       <c r="K265" s="31" t="n"/>
@@ -17046,7 +16840,7 @@
       <c r="A266" s="30" t="n"/>
       <c r="B266" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+041.04 - 0+058.81)</t>
+          <t>Caja de caida CC</t>
         </is>
       </c>
       <c r="C266" s="31" t="n">
@@ -17059,7 +16853,7 @@
       <c r="H266" s="31" t="n"/>
       <c r="I266" s="31" t="n"/>
       <c r="J266" s="31">
-        <f>'COLECTOR TRAMOS'!T26</f>
+        <f>'COLECTOR TRAMOS'!J35</f>
         <v/>
       </c>
       <c r="K266" s="31" t="n"/>
@@ -17069,7 +16863,7 @@
       <c r="A267" s="30" t="n"/>
       <c r="B267" s="30" t="inlineStr">
         <is>
-          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
+          <t>Bordes engrosados de abertura de registros</t>
         </is>
       </c>
       <c r="C267" s="31" t="n">
@@ -17082,7 +16876,7 @@
       <c r="H267" s="31" t="n"/>
       <c r="I267" s="31" t="n"/>
       <c r="J267" s="31">
-        <f>'COLECTOR TRAMOS'!T27</f>
+        <f>'COLECTOR TAPAS'!G20</f>
         <v/>
       </c>
       <c r="K267" s="31" t="n"/>
@@ -17092,11 +16886,11 @@
       <c r="A268" s="30" t="n"/>
       <c r="B268" s="30" t="inlineStr">
         <is>
-          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
+          <t>Descuento de aberturas de registro 0.70 x 0.70 x 0.10</t>
         </is>
       </c>
       <c r="C268" s="31" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D268" s="31" t="n"/>
       <c r="E268" s="31" t="n"/>
@@ -17105,40 +16899,46 @@
       <c r="H268" s="31" t="n"/>
       <c r="I268" s="31" t="n"/>
       <c r="J268" s="31">
-        <f>'COLECTOR TRAMOS'!T28</f>
+        <f>-'COLECTOR TAPAS'!$B$3*0.70*0.70*0.10</f>
         <v/>
       </c>
       <c r="K268" s="31" t="n"/>
       <c r="L268" s="30" t="n"/>
     </row>
     <row r="269">
-      <c r="A269" s="30" t="n"/>
-      <c r="B269" s="30" t="inlineStr">
-        <is>
-          <t>Caja de llegada CL</t>
-        </is>
-      </c>
-      <c r="C269" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D269" s="31" t="n"/>
-      <c r="E269" s="31" t="n"/>
-      <c r="F269" s="31" t="n"/>
-      <c r="G269" s="31" t="n"/>
-      <c r="H269" s="31" t="n"/>
-      <c r="I269" s="31" t="n"/>
-      <c r="J269" s="31">
-        <f>'COLECTOR TRAMOS'!J34</f>
-        <v/>
-      </c>
-      <c r="K269" s="31" t="n"/>
-      <c r="L269" s="30" t="n"/>
+      <c r="A269" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.04.04</t>
+        </is>
+      </c>
+      <c r="B269" s="28" t="inlineStr">
+        <is>
+          <t>ENCOFRADO Y DESENCOFRADO NORMAL EN COLECTOR Y CAJAS</t>
+        </is>
+      </c>
+      <c r="C269" s="29" t="n"/>
+      <c r="D269" s="29" t="n"/>
+      <c r="E269" s="29" t="n"/>
+      <c r="F269" s="29" t="n"/>
+      <c r="G269" s="29" t="n"/>
+      <c r="H269" s="29" t="n"/>
+      <c r="I269" s="29" t="n"/>
+      <c r="J269" s="29" t="n"/>
+      <c r="K269" s="29">
+        <f>SUM(J270:J278)</f>
+        <v/>
+      </c>
+      <c r="L269" s="28" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="30" t="n"/>
       <c r="B270" s="30" t="inlineStr">
         <is>
-          <t>Caja de caida CC</t>
+          <t>Tramo normal (0+000.00 - 0+026.32)</t>
         </is>
       </c>
       <c r="C270" s="31" t="n">
@@ -17151,7 +16951,7 @@
       <c r="H270" s="31" t="n"/>
       <c r="I270" s="31" t="n"/>
       <c r="J270" s="31">
-        <f>'COLECTOR TRAMOS'!J35</f>
+        <f>'COLECTOR TRAMOS'!U22</f>
         <v/>
       </c>
       <c r="K270" s="31" t="n"/>
@@ -17161,7 +16961,7 @@
       <c r="A271" s="30" t="n"/>
       <c r="B271" s="30" t="inlineStr">
         <is>
-          <t>Bordes engrosados de abertura de registros</t>
+          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
         </is>
       </c>
       <c r="C271" s="31" t="n">
@@ -17174,7 +16974,7 @@
       <c r="H271" s="31" t="n"/>
       <c r="I271" s="31" t="n"/>
       <c r="J271" s="31">
-        <f>'COLECTOR TAPAS'!G20</f>
+        <f>'COLECTOR TRAMOS'!U23</f>
         <v/>
       </c>
       <c r="K271" s="31" t="n"/>
@@ -17184,11 +16984,11 @@
       <c r="A272" s="30" t="n"/>
       <c r="B272" s="30" t="inlineStr">
         <is>
-          <t>Descuento de aberturas de registro 0.70 x 0.70 x 0.10</t>
+          <t>Tramo normal (0+031.33 - 0+039.04)</t>
         </is>
       </c>
       <c r="C272" s="31" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="D272" s="31" t="n"/>
       <c r="E272" s="31" t="n"/>
@@ -17197,46 +16997,40 @@
       <c r="H272" s="31" t="n"/>
       <c r="I272" s="31" t="n"/>
       <c r="J272" s="31">
-        <f>-'COLECTOR TAPAS'!$B$3*0.70*0.70*0.10</f>
+        <f>'COLECTOR TRAMOS'!U24</f>
         <v/>
       </c>
       <c r="K272" s="31" t="n"/>
       <c r="L272" s="30" t="n"/>
     </row>
     <row r="273">
-      <c r="A273" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.04.04</t>
-        </is>
-      </c>
-      <c r="B273" s="28" t="inlineStr">
-        <is>
-          <t>ENCOFRADO Y DESENCOFRADO NORMAL EN COLECTOR Y CAJAS</t>
-        </is>
-      </c>
-      <c r="C273" s="29" t="n"/>
-      <c r="D273" s="29" t="n"/>
-      <c r="E273" s="29" t="n"/>
-      <c r="F273" s="29" t="n"/>
-      <c r="G273" s="29" t="n"/>
-      <c r="H273" s="29" t="n"/>
-      <c r="I273" s="29" t="n"/>
-      <c r="J273" s="29" t="n"/>
-      <c r="K273" s="29">
-        <f>SUM(J274:J282)</f>
-        <v/>
-      </c>
-      <c r="L273" s="28" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
+      <c r="A273" s="30" t="n"/>
+      <c r="B273" s="30" t="inlineStr">
+        <is>
+          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
+        </is>
+      </c>
+      <c r="C273" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D273" s="31" t="n"/>
+      <c r="E273" s="31" t="n"/>
+      <c r="F273" s="31" t="n"/>
+      <c r="G273" s="31" t="n"/>
+      <c r="H273" s="31" t="n"/>
+      <c r="I273" s="31" t="n"/>
+      <c r="J273" s="31">
+        <f>'COLECTOR TRAMOS'!U25</f>
+        <v/>
+      </c>
+      <c r="K273" s="31" t="n"/>
+      <c r="L273" s="30" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="30" t="n"/>
       <c r="B274" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+000.00 - 0+026.32)</t>
+          <t>Tramo normal (0+041.04 - 0+058.81)</t>
         </is>
       </c>
       <c r="C274" s="31" t="n">
@@ -17249,7 +17043,7 @@
       <c r="H274" s="31" t="n"/>
       <c r="I274" s="31" t="n"/>
       <c r="J274" s="31">
-        <f>'COLECTOR TRAMOS'!U22</f>
+        <f>'COLECTOR TRAMOS'!U26</f>
         <v/>
       </c>
       <c r="K274" s="31" t="n"/>
@@ -17259,7 +17053,7 @@
       <c r="A275" s="30" t="n"/>
       <c r="B275" s="30" t="inlineStr">
         <is>
-          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
+          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
         </is>
       </c>
       <c r="C275" s="31" t="n">
@@ -17272,7 +17066,7 @@
       <c r="H275" s="31" t="n"/>
       <c r="I275" s="31" t="n"/>
       <c r="J275" s="31">
-        <f>'COLECTOR TRAMOS'!U23</f>
+        <f>'COLECTOR TRAMOS'!U27</f>
         <v/>
       </c>
       <c r="K275" s="31" t="n"/>
@@ -17282,7 +17076,7 @@
       <c r="A276" s="30" t="n"/>
       <c r="B276" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+031.33 - 0+039.04)</t>
+          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
         </is>
       </c>
       <c r="C276" s="31" t="n">
@@ -17295,7 +17089,7 @@
       <c r="H276" s="31" t="n"/>
       <c r="I276" s="31" t="n"/>
       <c r="J276" s="31">
-        <f>'COLECTOR TRAMOS'!U24</f>
+        <f>'COLECTOR TRAMOS'!U28</f>
         <v/>
       </c>
       <c r="K276" s="31" t="n"/>
@@ -17305,7 +17099,7 @@
       <c r="A277" s="30" t="n"/>
       <c r="B277" s="30" t="inlineStr">
         <is>
-          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
+          <t>Caja de llegada CL</t>
         </is>
       </c>
       <c r="C277" s="31" t="n">
@@ -17318,7 +17112,7 @@
       <c r="H277" s="31" t="n"/>
       <c r="I277" s="31" t="n"/>
       <c r="J277" s="31">
-        <f>'COLECTOR TRAMOS'!U25</f>
+        <f>'COLECTOR TRAMOS'!K34</f>
         <v/>
       </c>
       <c r="K277" s="31" t="n"/>
@@ -17328,7 +17122,7 @@
       <c r="A278" s="30" t="n"/>
       <c r="B278" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+041.04 - 0+058.81)</t>
+          <t>Caja de caida CC</t>
         </is>
       </c>
       <c r="C278" s="31" t="n">
@@ -17341,63 +17135,75 @@
       <c r="H278" s="31" t="n"/>
       <c r="I278" s="31" t="n"/>
       <c r="J278" s="31">
-        <f>'COLECTOR TRAMOS'!U26</f>
+        <f>'COLECTOR TRAMOS'!K35</f>
         <v/>
       </c>
       <c r="K278" s="31" t="n"/>
       <c r="L278" s="30" t="n"/>
     </row>
     <row r="279">
-      <c r="A279" s="30" t="n"/>
-      <c r="B279" s="30" t="inlineStr">
-        <is>
-          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
-        </is>
-      </c>
-      <c r="C279" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D279" s="31" t="n"/>
-      <c r="E279" s="31" t="n"/>
-      <c r="F279" s="31" t="n"/>
-      <c r="G279" s="31" t="n"/>
-      <c r="H279" s="31" t="n"/>
-      <c r="I279" s="31" t="n"/>
-      <c r="J279" s="31">
-        <f>'COLECTOR TRAMOS'!U27</f>
-        <v/>
-      </c>
-      <c r="K279" s="31" t="n"/>
-      <c r="L279" s="30" t="n"/>
+      <c r="A279" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.04.05</t>
+        </is>
+      </c>
+      <c r="B279" s="28" t="inlineStr">
+        <is>
+          <t>ACERO DE REFUERZO fy=4200 kg/cm2 EN COLECTOR Y CAJAS</t>
+        </is>
+      </c>
+      <c r="C279" s="29" t="n"/>
+      <c r="D279" s="29" t="n"/>
+      <c r="E279" s="29" t="n"/>
+      <c r="F279" s="29" t="n"/>
+      <c r="G279" s="29" t="n"/>
+      <c r="H279" s="29" t="n"/>
+      <c r="I279" s="29" t="n"/>
+      <c r="J279" s="29" t="n"/>
+      <c r="K279" s="29">
+        <f>+'COLECTOR ACERO'!H12</f>
+        <v/>
+      </c>
+      <c r="L279" s="28" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
     </row>
     <row r="280">
-      <c r="A280" s="30" t="n"/>
-      <c r="B280" s="30" t="inlineStr">
-        <is>
-          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
-        </is>
-      </c>
-      <c r="C280" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D280" s="31" t="n"/>
-      <c r="E280" s="31" t="n"/>
-      <c r="F280" s="31" t="n"/>
-      <c r="G280" s="31" t="n"/>
-      <c r="H280" s="31" t="n"/>
-      <c r="I280" s="31" t="n"/>
-      <c r="J280" s="31">
-        <f>'COLECTOR TRAMOS'!U28</f>
-        <v/>
-      </c>
-      <c r="K280" s="31" t="n"/>
-      <c r="L280" s="30" t="n"/>
+      <c r="A280" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.04.06</t>
+        </is>
+      </c>
+      <c r="B280" s="28" t="inlineStr">
+        <is>
+          <t>ACABADO FROTACHADO Y BRUÑADO DE LOSA SUPERIOR</t>
+        </is>
+      </c>
+      <c r="C280" s="29" t="n"/>
+      <c r="D280" s="29" t="n"/>
+      <c r="E280" s="29" t="n"/>
+      <c r="F280" s="29" t="n"/>
+      <c r="G280" s="29" t="n"/>
+      <c r="H280" s="29" t="n"/>
+      <c r="I280" s="29" t="n"/>
+      <c r="J280" s="29" t="n"/>
+      <c r="K280" s="29">
+        <f>SUM(J281:J289)</f>
+        <v/>
+      </c>
+      <c r="L280" s="28" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="30" t="n"/>
       <c r="B281" s="30" t="inlineStr">
         <is>
-          <t>Caja de llegada CL</t>
+          <t>Tramo normal (0+000.00 - 0+026.32)</t>
         </is>
       </c>
       <c r="C281" s="31" t="n">
@@ -17410,7 +17216,7 @@
       <c r="H281" s="31" t="n"/>
       <c r="I281" s="31" t="n"/>
       <c r="J281" s="31">
-        <f>'COLECTOR TRAMOS'!K34</f>
+        <f>'COLECTOR TRAMOS'!V22</f>
         <v/>
       </c>
       <c r="K281" s="31" t="n"/>
@@ -17420,7 +17226,7 @@
       <c r="A282" s="30" t="n"/>
       <c r="B282" s="30" t="inlineStr">
         <is>
-          <t>Caja de caida CC</t>
+          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
         </is>
       </c>
       <c r="C282" s="31" t="n">
@@ -17433,75 +17239,63 @@
       <c r="H282" s="31" t="n"/>
       <c r="I282" s="31" t="n"/>
       <c r="J282" s="31">
-        <f>'COLECTOR TRAMOS'!K35</f>
+        <f>'COLECTOR TRAMOS'!V23</f>
         <v/>
       </c>
       <c r="K282" s="31" t="n"/>
       <c r="L282" s="30" t="n"/>
     </row>
     <row r="283">
-      <c r="A283" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.04.05</t>
-        </is>
-      </c>
-      <c r="B283" s="28" t="inlineStr">
-        <is>
-          <t>ACERO DE REFUERZO fy=4200 kg/cm2 EN COLECTOR Y CAJAS</t>
-        </is>
-      </c>
-      <c r="C283" s="29" t="n"/>
-      <c r="D283" s="29" t="n"/>
-      <c r="E283" s="29" t="n"/>
-      <c r="F283" s="29" t="n"/>
-      <c r="G283" s="29" t="n"/>
-      <c r="H283" s="29" t="n"/>
-      <c r="I283" s="29" t="n"/>
-      <c r="J283" s="29" t="n"/>
-      <c r="K283" s="29">
-        <f>+'COLECTOR ACERO'!H13</f>
-        <v/>
-      </c>
-      <c r="L283" s="28" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
+      <c r="A283" s="30" t="n"/>
+      <c r="B283" s="30" t="inlineStr">
+        <is>
+          <t>Tramo normal (0+031.33 - 0+039.04)</t>
+        </is>
+      </c>
+      <c r="C283" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D283" s="31" t="n"/>
+      <c r="E283" s="31" t="n"/>
+      <c r="F283" s="31" t="n"/>
+      <c r="G283" s="31" t="n"/>
+      <c r="H283" s="31" t="n"/>
+      <c r="I283" s="31" t="n"/>
+      <c r="J283" s="31">
+        <f>'COLECTOR TRAMOS'!V24</f>
+        <v/>
+      </c>
+      <c r="K283" s="31" t="n"/>
+      <c r="L283" s="30" t="n"/>
     </row>
     <row r="284">
-      <c r="A284" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.04.06</t>
-        </is>
-      </c>
-      <c r="B284" s="28" t="inlineStr">
-        <is>
-          <t>ACABADO FROTACHADO Y BRUÑADO DE LOSA SUPERIOR</t>
-        </is>
-      </c>
-      <c r="C284" s="29" t="n"/>
-      <c r="D284" s="29" t="n"/>
-      <c r="E284" s="29" t="n"/>
-      <c r="F284" s="29" t="n"/>
-      <c r="G284" s="29" t="n"/>
-      <c r="H284" s="29" t="n"/>
-      <c r="I284" s="29" t="n"/>
-      <c r="J284" s="29" t="n"/>
-      <c r="K284" s="29">
-        <f>SUM(J285:J293)</f>
-        <v/>
-      </c>
-      <c r="L284" s="28" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
+      <c r="A284" s="30" t="n"/>
+      <c r="B284" s="30" t="inlineStr">
+        <is>
+          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
+        </is>
+      </c>
+      <c r="C284" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D284" s="31" t="n"/>
+      <c r="E284" s="31" t="n"/>
+      <c r="F284" s="31" t="n"/>
+      <c r="G284" s="31" t="n"/>
+      <c r="H284" s="31" t="n"/>
+      <c r="I284" s="31" t="n"/>
+      <c r="J284" s="31">
+        <f>'COLECTOR TRAMOS'!V25</f>
+        <v/>
+      </c>
+      <c r="K284" s="31" t="n"/>
+      <c r="L284" s="30" t="n"/>
     </row>
     <row r="285">
       <c r="A285" s="30" t="n"/>
       <c r="B285" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+000.00 - 0+026.32)</t>
+          <t>Tramo normal (0+041.04 - 0+058.81)</t>
         </is>
       </c>
       <c r="C285" s="31" t="n">
@@ -17514,7 +17308,7 @@
       <c r="H285" s="31" t="n"/>
       <c r="I285" s="31" t="n"/>
       <c r="J285" s="31">
-        <f>'COLECTOR TRAMOS'!V22</f>
+        <f>'COLECTOR TRAMOS'!V26</f>
         <v/>
       </c>
       <c r="K285" s="31" t="n"/>
@@ -17524,7 +17318,7 @@
       <c r="A286" s="30" t="n"/>
       <c r="B286" s="30" t="inlineStr">
         <is>
-          <t>Cruce de camiones (0+026.32 - 0+031.33)</t>
+          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
         </is>
       </c>
       <c r="C286" s="31" t="n">
@@ -17537,7 +17331,7 @@
       <c r="H286" s="31" t="n"/>
       <c r="I286" s="31" t="n"/>
       <c r="J286" s="31">
-        <f>'COLECTOR TRAMOS'!V23</f>
+        <f>'COLECTOR TRAMOS'!V27</f>
         <v/>
       </c>
       <c r="K286" s="31" t="n"/>
@@ -17547,7 +17341,7 @@
       <c r="A287" s="30" t="n"/>
       <c r="B287" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+031.33 - 0+039.04)</t>
+          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
         </is>
       </c>
       <c r="C287" s="31" t="n">
@@ -17560,7 +17354,7 @@
       <c r="H287" s="31" t="n"/>
       <c r="I287" s="31" t="n"/>
       <c r="J287" s="31">
-        <f>'COLECTOR TRAMOS'!V24</f>
+        <f>'COLECTOR TRAMOS'!V28</f>
         <v/>
       </c>
       <c r="K287" s="31" t="n"/>
@@ -17570,7 +17364,7 @@
       <c r="A288" s="30" t="n"/>
       <c r="B288" s="30" t="inlineStr">
         <is>
-          <t>Cruce de motos (0+039.04 - 0+041.04)</t>
+          <t>Caja de llegada CL</t>
         </is>
       </c>
       <c r="C288" s="31" t="n">
@@ -17583,7 +17377,7 @@
       <c r="H288" s="31" t="n"/>
       <c r="I288" s="31" t="n"/>
       <c r="J288" s="31">
-        <f>'COLECTOR TRAMOS'!V25</f>
+        <f>'COLECTOR TRAMOS'!M34</f>
         <v/>
       </c>
       <c r="K288" s="31" t="n"/>
@@ -17593,7 +17387,7 @@
       <c r="A289" s="30" t="n"/>
       <c r="B289" s="30" t="inlineStr">
         <is>
-          <t>Tramo normal (0+041.04 - 0+058.81)</t>
+          <t>Caja de caida CC</t>
         </is>
       </c>
       <c r="C289" s="31" t="n">
@@ -17606,40 +17400,46 @@
       <c r="H289" s="31" t="n"/>
       <c r="I289" s="31" t="n"/>
       <c r="J289" s="31">
-        <f>'COLECTOR TRAMOS'!V26</f>
+        <f>'COLECTOR TRAMOS'!M35</f>
         <v/>
       </c>
       <c r="K289" s="31" t="n"/>
       <c r="L289" s="30" t="n"/>
     </row>
     <row r="290">
-      <c r="A290" s="30" t="n"/>
-      <c r="B290" s="30" t="inlineStr">
-        <is>
-          <t>Tramo diagonal (quiebres) (0+058.81 - 0+066.89)</t>
-        </is>
-      </c>
-      <c r="C290" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D290" s="31" t="n"/>
-      <c r="E290" s="31" t="n"/>
-      <c r="F290" s="31" t="n"/>
-      <c r="G290" s="31" t="n"/>
-      <c r="H290" s="31" t="n"/>
-      <c r="I290" s="31" t="n"/>
-      <c r="J290" s="31">
-        <f>'COLECTOR TRAMOS'!V27</f>
-        <v/>
-      </c>
-      <c r="K290" s="31" t="n"/>
-      <c r="L290" s="30" t="n"/>
+      <c r="A290" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.04.07</t>
+        </is>
+      </c>
+      <c r="B290" s="28" t="inlineStr">
+        <is>
+          <t>CURADO DE CONCRETO EN COLECTOR Y CAJAS</t>
+        </is>
+      </c>
+      <c r="C290" s="29" t="n"/>
+      <c r="D290" s="29" t="n"/>
+      <c r="E290" s="29" t="n"/>
+      <c r="F290" s="29" t="n"/>
+      <c r="G290" s="29" t="n"/>
+      <c r="H290" s="29" t="n"/>
+      <c r="I290" s="29" t="n"/>
+      <c r="J290" s="29" t="n"/>
+      <c r="K290" s="29">
+        <f>SUM(J291:J292)</f>
+        <v/>
+      </c>
+      <c r="L290" s="28" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="30" t="n"/>
       <c r="B291" s="30" t="inlineStr">
         <is>
-          <t>Tramo recto final (0+066.89 - 0+069.89)</t>
+          <t>Losa superior (igual al acabado)</t>
         </is>
       </c>
       <c r="C291" s="31" t="n">
@@ -17652,7 +17452,7 @@
       <c r="H291" s="31" t="n"/>
       <c r="I291" s="31" t="n"/>
       <c r="J291" s="31">
-        <f>'COLECTOR TRAMOS'!V28</f>
+        <f>K280</f>
         <v/>
       </c>
       <c r="K291" s="31" t="n"/>
@@ -17662,7 +17462,7 @@
       <c r="A292" s="30" t="n"/>
       <c r="B292" s="30" t="inlineStr">
         <is>
-          <t>Caja de llegada CL</t>
+          <t>Caras exteriores de muros (2 x altura x longitud)</t>
         </is>
       </c>
       <c r="C292" s="31" t="n">
@@ -17675,44 +17475,43 @@
       <c r="H292" s="31" t="n"/>
       <c r="I292" s="31" t="n"/>
       <c r="J292" s="31">
-        <f>'COLECTOR TRAMOS'!M34</f>
+        <f>0.5*'COLECTOR TRAMOS'!U29</f>
         <v/>
       </c>
       <c r="K292" s="31" t="n"/>
       <c r="L292" s="30" t="n"/>
     </row>
     <row r="293">
-      <c r="A293" s="30" t="n"/>
-      <c r="B293" s="30" t="inlineStr">
-        <is>
-          <t>Caja de caida CC</t>
-        </is>
-      </c>
-      <c r="C293" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D293" s="31" t="n"/>
-      <c r="E293" s="31" t="n"/>
-      <c r="F293" s="31" t="n"/>
-      <c r="G293" s="31" t="n"/>
-      <c r="H293" s="31" t="n"/>
-      <c r="I293" s="31" t="n"/>
-      <c r="J293" s="31">
-        <f>'COLECTOR TRAMOS'!M35</f>
-        <v/>
-      </c>
-      <c r="K293" s="31" t="n"/>
-      <c r="L293" s="30" t="n"/>
+      <c r="A293" s="217" t="inlineStr">
+        <is>
+          <t>01.04.04.05</t>
+        </is>
+      </c>
+      <c r="B293" s="217" t="inlineStr">
+        <is>
+          <t>REGISTROS DE LIMPIEZA Y TAPAS</t>
+        </is>
+      </c>
+      <c r="C293" s="313" t="n"/>
+      <c r="D293" s="313" t="n"/>
+      <c r="E293" s="313" t="n"/>
+      <c r="F293" s="313" t="n"/>
+      <c r="G293" s="313" t="n"/>
+      <c r="H293" s="313" t="n"/>
+      <c r="I293" s="313" t="n"/>
+      <c r="J293" s="313" t="n"/>
+      <c r="K293" s="313" t="n"/>
+      <c r="L293" s="314" t="n"/>
     </row>
     <row r="294">
       <c r="A294" s="28" t="inlineStr">
         <is>
-          <t>01.04.04.04.07</t>
+          <t>01.04.04.05.01</t>
         </is>
       </c>
       <c r="B294" s="28" t="inlineStr">
         <is>
-          <t>CURADO DE CONCRETO EN COLECTOR Y CAJAS</t>
+          <t>CONTRAMARCO METALICO L 2"x2"x3/16" CON ANCLAJES</t>
         </is>
       </c>
       <c r="C294" s="29" t="n"/>
@@ -17724,92 +17523,111 @@
       <c r="I294" s="29" t="n"/>
       <c r="J294" s="29" t="n"/>
       <c r="K294" s="29">
-        <f>SUM(J295:J296)</f>
+        <f>+'COLECTOR TAPAS'!G15</f>
         <v/>
       </c>
       <c r="L294" s="28" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>und</t>
         </is>
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="30" t="n"/>
-      <c r="B295" s="30" t="inlineStr">
-        <is>
-          <t>Losa superior (igual al acabado)</t>
-        </is>
-      </c>
-      <c r="C295" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D295" s="31" t="n"/>
-      <c r="E295" s="31" t="n"/>
-      <c r="F295" s="31" t="n"/>
-      <c r="G295" s="31" t="n"/>
-      <c r="H295" s="31" t="n"/>
-      <c r="I295" s="31" t="n"/>
-      <c r="J295" s="31">
-        <f>K284</f>
-        <v/>
-      </c>
-      <c r="K295" s="31" t="n"/>
-      <c r="L295" s="30" t="n"/>
+      <c r="A295" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.05.02</t>
+        </is>
+      </c>
+      <c r="B295" s="28" t="inlineStr">
+        <is>
+          <t>MARCO METALICO DE TAPA L 1 1/2"x1 1/2"x1/8"</t>
+        </is>
+      </c>
+      <c r="C295" s="29" t="n"/>
+      <c r="D295" s="29" t="n"/>
+      <c r="E295" s="29" t="n"/>
+      <c r="F295" s="29" t="n"/>
+      <c r="G295" s="29" t="n"/>
+      <c r="H295" s="29" t="n"/>
+      <c r="I295" s="29" t="n"/>
+      <c r="J295" s="29" t="n"/>
+      <c r="K295" s="29">
+        <f>+'COLECTOR TAPAS'!G16</f>
+        <v/>
+      </c>
+      <c r="L295" s="28" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
     </row>
     <row r="296">
-      <c r="A296" s="30" t="n"/>
-      <c r="B296" s="30" t="inlineStr">
-        <is>
-          <t>Caras exteriores de muros (2 x altura x longitud)</t>
-        </is>
-      </c>
-      <c r="C296" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D296" s="31" t="n"/>
-      <c r="E296" s="31" t="n"/>
-      <c r="F296" s="31" t="n"/>
-      <c r="G296" s="31" t="n"/>
-      <c r="H296" s="31" t="n"/>
-      <c r="I296" s="31" t="n"/>
-      <c r="J296" s="31">
-        <f>0.5*'COLECTOR TRAMOS'!U29</f>
-        <v/>
-      </c>
-      <c r="K296" s="31" t="n"/>
-      <c r="L296" s="30" t="n"/>
+      <c r="A296" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.05.03</t>
+        </is>
+      </c>
+      <c r="B296" s="28" t="inlineStr">
+        <is>
+          <t>ANGULOS METALICOS P/MARCO Y CONTRAMARCO (incluye soldadura)</t>
+        </is>
+      </c>
+      <c r="C296" s="29" t="n"/>
+      <c r="D296" s="29" t="n"/>
+      <c r="E296" s="29" t="n"/>
+      <c r="F296" s="29" t="n"/>
+      <c r="G296" s="29" t="n"/>
+      <c r="H296" s="29" t="n"/>
+      <c r="I296" s="29" t="n"/>
+      <c r="J296" s="29" t="n"/>
+      <c r="K296" s="29">
+        <f>+'COLECTOR TAPAS'!G17</f>
+        <v/>
+      </c>
+      <c r="L296" s="28" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
     </row>
     <row r="297">
-      <c r="A297" s="217" t="inlineStr">
-        <is>
-          <t>01.04.04.05</t>
-        </is>
-      </c>
-      <c r="B297" s="217" t="inlineStr">
-        <is>
-          <t>REGISTROS DE LIMPIEZA Y TAPAS</t>
-        </is>
-      </c>
-      <c r="C297" s="313" t="n"/>
-      <c r="D297" s="313" t="n"/>
-      <c r="E297" s="313" t="n"/>
-      <c r="F297" s="313" t="n"/>
-      <c r="G297" s="313" t="n"/>
-      <c r="H297" s="313" t="n"/>
-      <c r="I297" s="313" t="n"/>
-      <c r="J297" s="313" t="n"/>
-      <c r="K297" s="313" t="n"/>
-      <c r="L297" s="314" t="n"/>
+      <c r="A297" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.05.04</t>
+        </is>
+      </c>
+      <c r="B297" s="28" t="inlineStr">
+        <is>
+          <t>TAPA DE CONCRETO ARMADO 0.68 x 0.68 x 0.08 m (incluye acero y asas)</t>
+        </is>
+      </c>
+      <c r="C297" s="29" t="n"/>
+      <c r="D297" s="29" t="n"/>
+      <c r="E297" s="29" t="n"/>
+      <c r="F297" s="29" t="n"/>
+      <c r="G297" s="29" t="n"/>
+      <c r="H297" s="29" t="n"/>
+      <c r="I297" s="29" t="n"/>
+      <c r="J297" s="29" t="n"/>
+      <c r="K297" s="29">
+        <f>+'COLECTOR TAPAS'!G18</f>
+        <v/>
+      </c>
+      <c r="L297" s="28" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="28" t="inlineStr">
         <is>
-          <t>01.04.04.05.01</t>
+          <t>01.04.04.05.05</t>
         </is>
       </c>
       <c r="B298" s="28" t="inlineStr">
         <is>
-          <t>CONTRAMARCO METALICO L 2"x2"x3/16" CON ANCLAJES</t>
+          <t>CONCRETO f'c=210 kg/cm2 EN TAPAS</t>
         </is>
       </c>
       <c r="C298" s="29" t="n"/>
@@ -17821,24 +17639,24 @@
       <c r="I298" s="29" t="n"/>
       <c r="J298" s="29" t="n"/>
       <c r="K298" s="29">
-        <f>+'COLECTOR TAPAS'!G15</f>
+        <f>+'COLECTOR TAPAS'!G19</f>
         <v/>
       </c>
       <c r="L298" s="28" t="inlineStr">
         <is>
-          <t>und</t>
+          <t>m³</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="28" t="inlineStr">
         <is>
-          <t>01.04.04.05.02</t>
+          <t>01.04.04.05.06</t>
         </is>
       </c>
       <c r="B299" s="28" t="inlineStr">
         <is>
-          <t>MARCO METALICO DE TAPA L 1 1/2"x1 1/2"x1/8"</t>
+          <t>ACERO DE REFUERZO fy=4200 kg/cm2 EN TAPAS, BORDES Y ANCLAJES</t>
         </is>
       </c>
       <c r="C299" s="29" t="n"/>
@@ -17850,24 +17668,24 @@
       <c r="I299" s="29" t="n"/>
       <c r="J299" s="29" t="n"/>
       <c r="K299" s="29">
-        <f>+'COLECTOR TAPAS'!G16</f>
+        <f>+'COLECTOR ACERO'!H13</f>
         <v/>
       </c>
       <c r="L299" s="28" t="inlineStr">
         <is>
-          <t>und</t>
+          <t>kg</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="28" t="inlineStr">
         <is>
-          <t>01.04.04.05.03</t>
+          <t>01.04.04.05.07</t>
         </is>
       </c>
       <c r="B300" s="28" t="inlineStr">
         <is>
-          <t>ANGULOS METALICOS P/MARCO Y CONTRAMARCO (incluye soldadura)</t>
+          <t>PINTURA ANTICORROSIVA Y ESMALTE EN ANGULOS</t>
         </is>
       </c>
       <c r="C300" s="29" t="n"/>
@@ -17879,53 +17697,46 @@
       <c r="I300" s="29" t="n"/>
       <c r="J300" s="29" t="n"/>
       <c r="K300" s="29">
-        <f>+'COLECTOR TAPAS'!G17</f>
+        <f>+'COLECTOR TAPAS'!G21</f>
         <v/>
       </c>
       <c r="L300" s="28" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m²</t>
         </is>
       </c>
     </row>
     <row r="301">
-      <c r="A301" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.05.04</t>
-        </is>
-      </c>
-      <c r="B301" s="28" t="inlineStr">
-        <is>
-          <t>TAPA DE CONCRETO ARMADO 0.68 x 0.68 x 0.08 m (incluye acero y asas)</t>
-        </is>
-      </c>
-      <c r="C301" s="29" t="n"/>
-      <c r="D301" s="29" t="n"/>
-      <c r="E301" s="29" t="n"/>
-      <c r="F301" s="29" t="n"/>
-      <c r="G301" s="29" t="n"/>
-      <c r="H301" s="29" t="n"/>
-      <c r="I301" s="29" t="n"/>
-      <c r="J301" s="29" t="n"/>
-      <c r="K301" s="29">
-        <f>+'COLECTOR TAPAS'!G18</f>
-        <v/>
-      </c>
-      <c r="L301" s="28" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
+      <c r="A301" s="217" t="inlineStr">
+        <is>
+          <t>01.04.04.06</t>
+        </is>
+      </c>
+      <c r="B301" s="217" t="inlineStr">
+        <is>
+          <t>JUNTAS Y EMPALMES</t>
+        </is>
+      </c>
+      <c r="C301" s="313" t="n"/>
+      <c r="D301" s="313" t="n"/>
+      <c r="E301" s="313" t="n"/>
+      <c r="F301" s="313" t="n"/>
+      <c r="G301" s="313" t="n"/>
+      <c r="H301" s="313" t="n"/>
+      <c r="I301" s="313" t="n"/>
+      <c r="J301" s="313" t="n"/>
+      <c r="K301" s="313" t="n"/>
+      <c r="L301" s="314" t="n"/>
     </row>
     <row r="302">
       <c r="A302" s="28" t="inlineStr">
         <is>
-          <t>01.04.04.05.05</t>
+          <t>01.04.04.06.01</t>
         </is>
       </c>
       <c r="B302" s="28" t="inlineStr">
         <is>
-          <t>CONCRETO f'c=210 kg/cm2 EN TAPAS</t>
+          <t>JUNTA DE DILATACION E=1" CON TECNOPOR Y SELLADOR ELASTOMERICO</t>
         </is>
       </c>
       <c r="C302" s="29" t="n"/>
@@ -17937,53 +17748,49 @@
       <c r="I302" s="29" t="n"/>
       <c r="J302" s="29" t="n"/>
       <c r="K302" s="29">
-        <f>+'COLECTOR TAPAS'!G19</f>
+        <f>SUM(J303:J303)</f>
         <v/>
       </c>
       <c r="L302" s="28" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.05.06</t>
-        </is>
-      </c>
-      <c r="B303" s="28" t="inlineStr">
-        <is>
-          <t>ACERO DE REFUERZO fy=4200 kg/cm2 EN TAPAS, BORDES Y ANCLAJES</t>
-        </is>
-      </c>
-      <c r="C303" s="29" t="n"/>
-      <c r="D303" s="29" t="n"/>
-      <c r="E303" s="29" t="n"/>
-      <c r="F303" s="29" t="n"/>
-      <c r="G303" s="29" t="n"/>
-      <c r="H303" s="29" t="n"/>
-      <c r="I303" s="29" t="n"/>
-      <c r="J303" s="29" t="n"/>
-      <c r="K303" s="29">
-        <f>+'COLECTOR ACERO'!H14</f>
-        <v/>
-      </c>
-      <c r="L303" s="28" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
+      <c r="A303" s="30" t="n"/>
+      <c r="B303" s="30" t="inlineStr">
+        <is>
+          <t>Juntas cada 4.00 m (perimetro de la seccion)</t>
+        </is>
+      </c>
+      <c r="C303" s="31" t="n">
+        <v>17</v>
+      </c>
+      <c r="D303" s="31" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="E303" s="31" t="n"/>
+      <c r="F303" s="31" t="n"/>
+      <c r="G303" s="31" t="n"/>
+      <c r="H303" s="31" t="n"/>
+      <c r="I303" s="31" t="n"/>
+      <c r="J303" s="31">
+        <f>C303*D303</f>
+        <v/>
+      </c>
+      <c r="K303" s="31" t="n"/>
+      <c r="L303" s="30" t="n"/>
     </row>
     <row r="304">
       <c r="A304" s="28" t="inlineStr">
         <is>
-          <t>01.04.04.05.07</t>
+          <t>01.04.04.06.02</t>
         </is>
       </c>
       <c r="B304" s="28" t="inlineStr">
         <is>
-          <t>PINTURA ANTICORROSIVA Y ESMALTE EN ANGULOS</t>
+          <t>JUNTA DE TECNOPOR E=1" ENTRE COLECTOR, CERCO Y PISO ADYACENTE</t>
         </is>
       </c>
       <c r="C304" s="29" t="n"/>
@@ -17995,475 +17802,116 @@
       <c r="I304" s="29" t="n"/>
       <c r="J304" s="29" t="n"/>
       <c r="K304" s="29">
-        <f>+'COLECTOR TAPAS'!G21</f>
+        <f>SUM(J305:J306)</f>
         <v/>
       </c>
       <c r="L304" s="28" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m</t>
         </is>
       </c>
     </row>
     <row r="305">
-      <c r="A305" s="217" t="inlineStr">
-        <is>
-          <t>01.04.04.06</t>
-        </is>
-      </c>
-      <c r="B305" s="217" t="inlineStr">
-        <is>
-          <t>JUNTAS, EMPALMES Y PROLONGACION DE CUNETAS</t>
-        </is>
-      </c>
-      <c r="C305" s="313" t="n"/>
-      <c r="D305" s="313" t="n"/>
-      <c r="E305" s="313" t="n"/>
-      <c r="F305" s="313" t="n"/>
-      <c r="G305" s="313" t="n"/>
-      <c r="H305" s="313" t="n"/>
-      <c r="I305" s="313" t="n"/>
-      <c r="J305" s="313" t="n"/>
-      <c r="K305" s="313" t="n"/>
-      <c r="L305" s="314" t="n"/>
+      <c r="A305" s="30" t="n"/>
+      <c r="B305" s="30" t="inlineStr">
+        <is>
+          <t>Contra el cimiento del cerco (tramo pegado al cerco)</t>
+        </is>
+      </c>
+      <c r="C305" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D305" s="31" t="n">
+        <v>58.81</v>
+      </c>
+      <c r="E305" s="31" t="n"/>
+      <c r="F305" s="31" t="n"/>
+      <c r="G305" s="31" t="n"/>
+      <c r="H305" s="31" t="n"/>
+      <c r="I305" s="31" t="n"/>
+      <c r="J305" s="31">
+        <f>C305*D305</f>
+        <v/>
+      </c>
+      <c r="K305" s="31" t="n"/>
+      <c r="L305" s="30" t="n"/>
     </row>
     <row r="306">
-      <c r="A306" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.06.01</t>
-        </is>
-      </c>
-      <c r="B306" s="28" t="inlineStr">
-        <is>
-          <t>JUNTA DE DILATACION E=1" CON TECNOPOR Y SELLADOR ELASTOMERICO</t>
-        </is>
-      </c>
-      <c r="C306" s="29" t="n"/>
-      <c r="D306" s="29" t="n"/>
-      <c r="E306" s="29" t="n"/>
-      <c r="F306" s="29" t="n"/>
-      <c r="G306" s="29" t="n"/>
-      <c r="H306" s="29" t="n"/>
-      <c r="I306" s="29" t="n"/>
-      <c r="J306" s="29" t="n"/>
-      <c r="K306" s="29">
-        <f>SUM(J307:J307)</f>
-        <v/>
-      </c>
-      <c r="L306" s="28" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
+      <c r="A306" s="30" t="n"/>
+      <c r="B306" s="30" t="inlineStr">
+        <is>
+          <t>Borde de losa con el piso adyacente (ambos lados, colector y cajas)</t>
+        </is>
+      </c>
+      <c r="C306" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D306" s="31" t="n">
+        <v>150.97</v>
+      </c>
+      <c r="E306" s="31" t="n"/>
+      <c r="F306" s="31" t="n"/>
+      <c r="G306" s="31" t="n"/>
+      <c r="H306" s="31" t="n"/>
+      <c r="I306" s="31" t="n"/>
+      <c r="J306" s="31">
+        <f>C306*D306</f>
+        <v/>
+      </c>
+      <c r="K306" s="31" t="n"/>
+      <c r="L306" s="30" t="n"/>
     </row>
     <row r="307">
-      <c r="A307" s="30" t="n"/>
-      <c r="B307" s="30" t="inlineStr">
-        <is>
-          <t>Juntas cada 4.00 m (perimetro de la seccion)</t>
-        </is>
-      </c>
-      <c r="C307" s="31" t="n">
-        <v>17</v>
-      </c>
-      <c r="D307" s="31" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="E307" s="31" t="n"/>
-      <c r="F307" s="31" t="n"/>
-      <c r="G307" s="31" t="n"/>
-      <c r="H307" s="31" t="n"/>
-      <c r="I307" s="31" t="n"/>
-      <c r="J307" s="31">
-        <f>C307*D307</f>
-        <v/>
-      </c>
-      <c r="K307" s="31" t="n"/>
-      <c r="L307" s="30" t="n"/>
+      <c r="A307" s="28" t="inlineStr">
+        <is>
+          <t>01.04.04.06.03</t>
+        </is>
+      </c>
+      <c r="B307" s="28" t="inlineStr">
+        <is>
+          <t>EMPALME DE CUNETA AL COLECTOR (ventana en muro y caida)</t>
+        </is>
+      </c>
+      <c r="C307" s="29" t="n"/>
+      <c r="D307" s="29" t="n"/>
+      <c r="E307" s="29" t="n"/>
+      <c r="F307" s="29" t="n"/>
+      <c r="G307" s="29" t="n"/>
+      <c r="H307" s="29" t="n"/>
+      <c r="I307" s="29" t="n"/>
+      <c r="J307" s="29" t="n"/>
+      <c r="K307" s="29">
+        <f>SUM(J308:J308)</f>
+        <v/>
+      </c>
+      <c r="L307" s="28" t="inlineStr">
+        <is>
+          <t>und</t>
+        </is>
+      </c>
     </row>
     <row r="308">
-      <c r="A308" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.06.02</t>
-        </is>
-      </c>
-      <c r="B308" s="28" t="inlineStr">
-        <is>
-          <t>JUNTA DE TECNOPOR E=1" ENTRE COLECTOR, CERCO Y PISO ADYACENTE</t>
-        </is>
-      </c>
-      <c r="C308" s="29" t="n"/>
-      <c r="D308" s="29" t="n"/>
-      <c r="E308" s="29" t="n"/>
-      <c r="F308" s="29" t="n"/>
-      <c r="G308" s="29" t="n"/>
-      <c r="H308" s="29" t="n"/>
-      <c r="I308" s="29" t="n"/>
-      <c r="J308" s="29" t="n"/>
-      <c r="K308" s="29">
-        <f>SUM(J309:J310)</f>
-        <v/>
-      </c>
-      <c r="L308" s="28" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" s="30" t="n"/>
-      <c r="B309" s="30" t="inlineStr">
-        <is>
-          <t>Contra el cimiento del cerco (tramo pegado al cerco)</t>
-        </is>
-      </c>
-      <c r="C309" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D309" s="31" t="n">
-        <v>58.81</v>
-      </c>
-      <c r="E309" s="31" t="n"/>
-      <c r="F309" s="31" t="n"/>
-      <c r="G309" s="31" t="n"/>
-      <c r="H309" s="31" t="n"/>
-      <c r="I309" s="31" t="n"/>
-      <c r="J309" s="31">
-        <f>C309*D309</f>
-        <v/>
-      </c>
-      <c r="K309" s="31" t="n"/>
-      <c r="L309" s="30" t="n"/>
-    </row>
-    <row r="310">
-      <c r="A310" s="30" t="n"/>
-      <c r="B310" s="30" t="inlineStr">
-        <is>
-          <t>Borde de losa con el piso adyacente (ambos lados, colector y cajas)</t>
-        </is>
-      </c>
-      <c r="C310" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D310" s="31" t="n">
-        <v>150.97</v>
-      </c>
-      <c r="E310" s="31" t="n"/>
-      <c r="F310" s="31" t="n"/>
-      <c r="G310" s="31" t="n"/>
-      <c r="H310" s="31" t="n"/>
-      <c r="I310" s="31" t="n"/>
-      <c r="J310" s="31">
-        <f>C310*D310</f>
-        <v/>
-      </c>
-      <c r="K310" s="31" t="n"/>
-      <c r="L310" s="30" t="n"/>
-    </row>
-    <row r="311">
-      <c r="A311" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.06.03</t>
-        </is>
-      </c>
-      <c r="B311" s="28" t="inlineStr">
-        <is>
-          <t>EMPALME DE CUNETA AL COLECTOR (ventana en muro y caida)</t>
-        </is>
-      </c>
-      <c r="C311" s="29" t="n"/>
-      <c r="D311" s="29" t="n"/>
-      <c r="E311" s="29" t="n"/>
-      <c r="F311" s="29" t="n"/>
-      <c r="G311" s="29" t="n"/>
-      <c r="H311" s="29" t="n"/>
-      <c r="I311" s="29" t="n"/>
-      <c r="J311" s="29" t="n"/>
-      <c r="K311" s="29">
-        <f>SUM(J312:J312)</f>
-        <v/>
-      </c>
-      <c r="L311" s="28" t="inlineStr">
-        <is>
-          <t>und</t>
-        </is>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" s="30" t="n"/>
-      <c r="B312" s="30" t="inlineStr">
+      <c r="A308" s="30" t="n"/>
+      <c r="B308" s="30" t="inlineStr">
         <is>
           <t>Cunetas Ejes 01, 02, 06, 07, 11 y 12</t>
         </is>
       </c>
-      <c r="C312" s="31" t="n">
+      <c r="C308" s="31" t="n">
         <v>6</v>
       </c>
-      <c r="D312" s="31" t="n"/>
-      <c r="E312" s="31" t="n"/>
-      <c r="F312" s="31" t="n"/>
-      <c r="G312" s="31" t="n"/>
-      <c r="H312" s="31" t="n"/>
-      <c r="I312" s="31" t="n"/>
-      <c r="J312" s="31">
-        <f>C312</f>
-        <v/>
-      </c>
-      <c r="K312" s="31" t="n"/>
-      <c r="L312" s="30" t="n"/>
-    </row>
-    <row r="313">
-      <c r="A313" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.06.04</t>
-        </is>
-      </c>
-      <c r="B313" s="28" t="inlineStr">
-        <is>
-          <t>CONCRETO f'c=210 kg/cm2 EN PROLONGACION DE CUNETAS 0.40 x H</t>
-        </is>
-      </c>
-      <c r="C313" s="29" t="n"/>
-      <c r="D313" s="29" t="n"/>
-      <c r="E313" s="29" t="n"/>
-      <c r="F313" s="29" t="n"/>
-      <c r="G313" s="29" t="n"/>
-      <c r="H313" s="29" t="n"/>
-      <c r="I313" s="29" t="n"/>
-      <c r="J313" s="29" t="n"/>
-      <c r="K313" s="29">
-        <f>SUM(J314:J315)</f>
-        <v/>
-      </c>
-      <c r="L313" s="28" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" s="30" t="n"/>
-      <c r="B314" s="30" t="inlineStr">
-        <is>
-          <t>Prolongacion cuneta Eje 11</t>
-        </is>
-      </c>
-      <c r="C314" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D314" s="31" t="n"/>
-      <c r="E314" s="31" t="n"/>
-      <c r="F314" s="31" t="n"/>
-      <c r="G314" s="31" t="n"/>
-      <c r="H314" s="31" t="n"/>
-      <c r="I314" s="31" t="n"/>
-      <c r="J314" s="31">
-        <f>'COLECTOR TRAMOS'!I36</f>
-        <v/>
-      </c>
-      <c r="K314" s="31" t="n"/>
-      <c r="L314" s="30" t="n"/>
-    </row>
-    <row r="315">
-      <c r="A315" s="30" t="n"/>
-      <c r="B315" s="30" t="inlineStr">
-        <is>
-          <t>Prolongacion cuneta Eje 12</t>
-        </is>
-      </c>
-      <c r="C315" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D315" s="31" t="n"/>
-      <c r="E315" s="31" t="n"/>
-      <c r="F315" s="31" t="n"/>
-      <c r="G315" s="31" t="n"/>
-      <c r="H315" s="31" t="n"/>
-      <c r="I315" s="31" t="n"/>
-      <c r="J315" s="31">
-        <f>'COLECTOR TRAMOS'!I37</f>
-        <v/>
-      </c>
-      <c r="K315" s="31" t="n"/>
-      <c r="L315" s="30" t="n"/>
-    </row>
-    <row r="316">
-      <c r="A316" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.06.05</t>
-        </is>
-      </c>
-      <c r="B316" s="28" t="inlineStr">
-        <is>
-          <t>ENCOFRADO Y DESENCOFRADO EN PROLONGACION DE CUNETAS</t>
-        </is>
-      </c>
-      <c r="C316" s="29" t="n"/>
-      <c r="D316" s="29" t="n"/>
-      <c r="E316" s="29" t="n"/>
-      <c r="F316" s="29" t="n"/>
-      <c r="G316" s="29" t="n"/>
-      <c r="H316" s="29" t="n"/>
-      <c r="I316" s="29" t="n"/>
-      <c r="J316" s="29" t="n"/>
-      <c r="K316" s="29">
-        <f>SUM(J317:J318)</f>
-        <v/>
-      </c>
-      <c r="L316" s="28" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" s="30" t="n"/>
-      <c r="B317" s="30" t="inlineStr">
-        <is>
-          <t>Prolongacion cuneta Eje 11</t>
-        </is>
-      </c>
-      <c r="C317" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D317" s="31" t="n"/>
-      <c r="E317" s="31" t="n"/>
-      <c r="F317" s="31" t="n"/>
-      <c r="G317" s="31" t="n"/>
-      <c r="H317" s="31" t="n"/>
-      <c r="I317" s="31" t="n"/>
-      <c r="J317" s="31">
-        <f>'COLECTOR TRAMOS'!K36</f>
-        <v/>
-      </c>
-      <c r="K317" s="31" t="n"/>
-      <c r="L317" s="30" t="n"/>
-    </row>
-    <row r="318">
-      <c r="A318" s="30" t="n"/>
-      <c r="B318" s="30" t="inlineStr">
-        <is>
-          <t>Prolongacion cuneta Eje 12</t>
-        </is>
-      </c>
-      <c r="C318" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D318" s="31" t="n"/>
-      <c r="E318" s="31" t="n"/>
-      <c r="F318" s="31" t="n"/>
-      <c r="G318" s="31" t="n"/>
-      <c r="H318" s="31" t="n"/>
-      <c r="I318" s="31" t="n"/>
-      <c r="J318" s="31">
-        <f>'COLECTOR TRAMOS'!K37</f>
-        <v/>
-      </c>
-      <c r="K318" s="31" t="n"/>
-      <c r="L318" s="30" t="n"/>
-    </row>
-    <row r="319">
-      <c r="A319" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.06.06</t>
-        </is>
-      </c>
-      <c r="B319" s="28" t="inlineStr">
-        <is>
-          <t>ACERO DE REFUERZO fy=4200 kg/cm2 EN PROLONGACION DE CUNETAS</t>
-        </is>
-      </c>
-      <c r="C319" s="29" t="n"/>
-      <c r="D319" s="29" t="n"/>
-      <c r="E319" s="29" t="n"/>
-      <c r="F319" s="29" t="n"/>
-      <c r="G319" s="29" t="n"/>
-      <c r="H319" s="29" t="n"/>
-      <c r="I319" s="29" t="n"/>
-      <c r="J319" s="29" t="n"/>
-      <c r="K319" s="29">
-        <f>+'COLECTOR ACERO'!H15</f>
-        <v/>
-      </c>
-      <c r="L319" s="28" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" s="28" t="inlineStr">
-        <is>
-          <t>01.04.04.06.07</t>
-        </is>
-      </c>
-      <c r="B320" s="28" t="inlineStr">
-        <is>
-          <t>TAPA DE CONCRETO EN PROLONGACION DE CUNETAS (losa 0.60 x 0.08)</t>
-        </is>
-      </c>
-      <c r="C320" s="29" t="n"/>
-      <c r="D320" s="29" t="n"/>
-      <c r="E320" s="29" t="n"/>
-      <c r="F320" s="29" t="n"/>
-      <c r="G320" s="29" t="n"/>
-      <c r="H320" s="29" t="n"/>
-      <c r="I320" s="29" t="n"/>
-      <c r="J320" s="29" t="n"/>
-      <c r="K320" s="29">
-        <f>SUM(J321:J322)</f>
-        <v/>
-      </c>
-      <c r="L320" s="28" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" s="30" t="n"/>
-      <c r="B321" s="30" t="inlineStr">
-        <is>
-          <t>Prolongacion cuneta Eje 11</t>
-        </is>
-      </c>
-      <c r="C321" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D321" s="31" t="n"/>
-      <c r="E321" s="31" t="n"/>
-      <c r="F321" s="31" t="n"/>
-      <c r="G321" s="31" t="n"/>
-      <c r="H321" s="31" t="n"/>
-      <c r="I321" s="31" t="n"/>
-      <c r="J321" s="31">
-        <f>'COLECTOR TRAMOS'!M36</f>
-        <v/>
-      </c>
-      <c r="K321" s="31" t="n"/>
-      <c r="L321" s="30" t="n"/>
-    </row>
-    <row r="322">
-      <c r="A322" s="30" t="n"/>
-      <c r="B322" s="30" t="inlineStr">
-        <is>
-          <t>Prolongacion cuneta Eje 12</t>
-        </is>
-      </c>
-      <c r="C322" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="D322" s="31" t="n"/>
-      <c r="E322" s="31" t="n"/>
-      <c r="F322" s="31" t="n"/>
-      <c r="G322" s="31" t="n"/>
-      <c r="H322" s="31" t="n"/>
-      <c r="I322" s="31" t="n"/>
-      <c r="J322" s="31">
-        <f>'COLECTOR TRAMOS'!M37</f>
-        <v/>
-      </c>
-      <c r="K322" s="31" t="n"/>
-      <c r="L322" s="30" t="n"/>
+      <c r="D308" s="31" t="n"/>
+      <c r="E308" s="31" t="n"/>
+      <c r="F308" s="31" t="n"/>
+      <c r="G308" s="31" t="n"/>
+      <c r="H308" s="31" t="n"/>
+      <c r="I308" s="31" t="n"/>
+      <c r="J308" s="31">
+        <f>C308</f>
+        <v/>
+      </c>
+      <c r="K308" s="31" t="n"/>
+      <c r="L308" s="30" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="12">

</xml_diff>

<commit_message>
Planilla: la imagen de encabezado se reinyecta despues de los saltos de pagina (orden del esquema), Excel ya no vacia las hojas CONCRETO EN CUNETAS y ENCOFRADO
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables/METRADO_DRENAJE_PLUVIAL_MUJERES_VIOLENTADAS_CON_COLECTOR.xlsx
+++ b/entregables/METRADO_DRENAJE_PLUVIAL_MUJERES_VIOLENTADAS_CON_COLECTOR.xlsx
@@ -27498,10 +27498,10 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <legacyDrawingHF r:id="rIdHF1"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="143" min="0" max="15" man="1"/>
   </rowBreaks>
+  <legacyDrawingHF r:id="rIdHF1"/>
 </worksheet>
 </file>
 
@@ -30269,10 +30269,10 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
-  <legacyDrawingHF r:id="rIdHF1"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="80" min="0" max="15" man="1"/>
   </rowBreaks>
+  <legacyDrawingHF r:id="rIdHF1"/>
 </worksheet>
 </file>
 

</xml_diff>